<commit_message>
feat: add more script
</commit_message>
<xml_diff>
--- a/data/all_component_analysis.xlsx
+++ b/data/all_component_analysis.xlsx
@@ -838,7 +838,7 @@
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>P-body</t>
+          <t>kinetochore</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -848,7 +848,7 @@
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>kinetochore</t>
+          <t>P-body</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1298,7 +1298,7 @@
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>cell surface</t>
+          <t>catalytic step 2 spliceosome</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -1308,7 +1308,7 @@
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>catalytic step 2 spliceosome</t>
+          <t>cell surface</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -1328,7 +1328,7 @@
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>polysome</t>
+          <t>condensed nuclear chromosome</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -1338,7 +1338,7 @@
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>condensed nuclear chromosome</t>
+          <t>polysome</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -1418,7 +1418,7 @@
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t>nuclear pore outer ring</t>
+          <t>eisosome</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -1428,7 +1428,7 @@
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t>eisosome</t>
+          <t>nuclear pore outer ring</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -1478,7 +1478,7 @@
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t>extracellular space</t>
+          <t>peroxisomal matrix</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -1488,7 +1488,7 @@
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t>peroxisomal matrix</t>
+          <t>extracellular space</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -1518,7 +1518,7 @@
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t>cell septum</t>
+          <t>perinuclear region of cytoplasm</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -1528,7 +1528,7 @@
     <row r="111">
       <c r="A111" s="1" t="inlineStr">
         <is>
-          <t>perinuclear region of cytoplasm</t>
+          <t>cell septum</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -1548,7 +1548,7 @@
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t>endoplasmic reticulum lumen</t>
+          <t>proteasome storage granule</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -1568,7 +1568,7 @@
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>proteasome storage granule</t>
+          <t>endoplasmic reticulum lumen</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -1578,7 +1578,7 @@
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>replication fork</t>
+          <t>ER to Golgi transport vesicle membrane</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -1588,7 +1588,7 @@
     <row r="117">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>ER to Golgi transport vesicle membrane</t>
+          <t>nucleosome</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -1598,7 +1598,7 @@
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>microtubule plus-end</t>
+          <t>replication fork</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -1608,7 +1608,7 @@
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>nucleosome</t>
+          <t>microtubule plus-end</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -1688,7 +1688,7 @@
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>condensed chromosome, centromeric region</t>
+          <t>U2-type catalytic step 2 spliceosome</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -1698,7 +1698,7 @@
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>U2-type catalytic step 2 spliceosome</t>
+          <t>cellular bud neck contractile ring</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -1708,7 +1708,7 @@
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>cellular bud neck contractile ring</t>
+          <t>condensed chromosome, centromeric region</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -1718,7 +1718,7 @@
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>fungal-type vacuole lumen</t>
+          <t>multivesicular body</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -1728,7 +1728,7 @@
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>multivesicular body</t>
+          <t>late endosome membrane</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -1738,7 +1738,7 @@
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>late endosome membrane</t>
+          <t>ascospore wall</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -1748,7 +1748,7 @@
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>ascospore wall</t>
+          <t>cellular bud neck septin ring</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -1758,7 +1758,7 @@
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>cellular bud neck septin ring</t>
+          <t>fungal-type vacuole lumen</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -1768,7 +1768,7 @@
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>intrinsic component of membrane</t>
+          <t>recycling endosome</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -1778,7 +1778,7 @@
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>perinuclear endoplasmic reticulum</t>
+          <t>intrinsic component of membrane</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -1788,7 +1788,7 @@
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>nuclear chromosome</t>
+          <t>microtubule organizing center</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -1798,7 +1798,7 @@
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>microtubule organizing center</t>
+          <t>nuclear chromosome</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -1808,7 +1808,7 @@
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>recycling endosome</t>
+          <t>perinuclear endoplasmic reticulum</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -1818,7 +1818,7 @@
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>cellular bud scar</t>
+          <t>nuclear replication fork</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -1828,7 +1828,7 @@
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>nuclear replication fork</t>
+          <t>cellular bud scar</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -1848,7 +1848,7 @@
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>nuclear outer membrane-endoplasmic reticulum membrane network</t>
+          <t>mitochondrial envelope</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -1858,7 +1858,7 @@
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>mitochondrial envelope</t>
+          <t>nuclear outer membrane-endoplasmic reticulum membrane network</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -1898,7 +1898,7 @@
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>nuclear pore cytoplasmic filaments</t>
+          <t>vacuolar proton-transporting V-type ATPase, V1 domain</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -1908,7 +1908,7 @@
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>vacuolar proton-transporting V-type ATPase, V1 domain</t>
+          <t>nuclear pore cytoplasmic filaments</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -1918,7 +1918,7 @@
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>integral component of mitochondrial membrane</t>
+          <t>cell cortex of cell tip</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -1928,7 +1928,7 @@
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>cell cortex of cell tip</t>
+          <t>endocytic vesicle</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -1938,7 +1938,7 @@
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>endocytic vesicle</t>
+          <t>integral component of mitochondrial membrane</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -1948,7 +1948,7 @@
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>cytoplasmic vesicle membrane</t>
+          <t>respirasome</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -1958,7 +1958,7 @@
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>transcriptionally active chromatin</t>
+          <t>cytoplasmic vesicle membrane</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -1968,7 +1968,7 @@
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>respirasome</t>
+          <t>transcriptionally active chromatin</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -1978,7 +1978,7 @@
     <row r="156">
       <c r="A156" s="1" t="inlineStr">
         <is>
-          <t>membrane coat</t>
+          <t>CHRAC</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -1988,7 +1988,7 @@
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>vacuolar proton-transporting V-type ATPase, V0 domain</t>
+          <t>membrane coat</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -1998,7 +1998,7 @@
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>CHRAC</t>
+          <t>vacuolar proton-transporting V-type ATPase, V0 domain</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -2008,7 +2008,7 @@
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>vacuole-mitochondrion membrane contact site</t>
+          <t>cytoophidium</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -2028,7 +2028,7 @@
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>cytoophidium</t>
+          <t>nuclear pore nuclear basket</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -2048,7 +2048,7 @@
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>nuclear pore nuclear basket</t>
+          <t>vacuole-mitochondrion membrane contact site</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -2088,7 +2088,7 @@
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>transport vesicle</t>
+          <t>COPI-coated vesicle membrane</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -2098,7 +2098,7 @@
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>extrinsic component of endoplasmic reticulum membrane</t>
+          <t>transport vesicle</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -2118,7 +2118,7 @@
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>COPI-coated vesicle membrane</t>
+          <t>extrinsic component of endoplasmic reticulum membrane</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -2158,7 +2158,7 @@
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t>Golgi lumen</t>
+          <t>equatorial microtubule organizing center</t>
         </is>
       </c>
       <c r="B174" t="n">
@@ -2168,7 +2168,7 @@
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>equatorial microtubule organizing center</t>
+          <t>Golgi lumen</t>
         </is>
       </c>
       <c r="B175" t="n">
@@ -2178,7 +2178,7 @@
     <row r="176">
       <c r="A176" s="1" t="inlineStr">
         <is>
-          <t>endoplasmic reticulum tubular network</t>
+          <t>mating projection</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -2188,7 +2188,7 @@
     <row r="177">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>intrinsic component of mitochondrial inner membrane</t>
+          <t>growing cell tip</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -2198,7 +2198,7 @@
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>vacuole-isolation membrane contact site</t>
+          <t>Golgi trans cisterna</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -2208,7 +2208,7 @@
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>mitochondrial crista junction</t>
+          <t>clathrin-coated vesicle membrane</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -2218,7 +2218,7 @@
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>Golgi cis cisterna</t>
+          <t>early endosome membrane</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -2228,7 +2228,7 @@
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>Golgi trans cisterna</t>
+          <t>mitochondrial proton-transporting ATP synthase, stator stalk</t>
         </is>
       </c>
       <c r="B181" t="n">
@@ -2238,7 +2238,7 @@
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>growing cell tip</t>
+          <t>endoplasmic reticulum tubular network</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -2248,7 +2248,7 @@
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>mitochondrial proton-transporting ATP synthase, stator stalk</t>
+          <t>Golgi cis cisterna</t>
         </is>
       </c>
       <c r="B183" t="n">
@@ -2258,7 +2258,7 @@
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>proton-transporting V-type ATPase, V0 domain</t>
+          <t>vacuole-isolation membrane contact site</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -2268,7 +2268,7 @@
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>clathrin-coated vesicle membrane</t>
+          <t>phagophore</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -2278,7 +2278,7 @@
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>mating projection</t>
+          <t>mitochondrial crista junction</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -2288,7 +2288,7 @@
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>early endosome membrane</t>
+          <t>proton-transporting V-type ATPase, V0 domain</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -2298,7 +2298,7 @@
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>phagophore</t>
+          <t>intrinsic component of mitochondrial inner membrane</t>
         </is>
       </c>
       <c r="B188" t="n">
@@ -2308,7 +2308,7 @@
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>mitochondrial respirasome</t>
+          <t>prospore membrane leading edge</t>
         </is>
       </c>
       <c r="B189" t="n">
@@ -2318,7 +2318,7 @@
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>signal recognition particle</t>
+          <t>condensed chromosome</t>
         </is>
       </c>
       <c r="B190" t="n">
@@ -2328,7 +2328,7 @@
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>condensed chromosome</t>
+          <t>cytosolic ribosome</t>
         </is>
       </c>
       <c r="B191" t="n">
@@ -2348,7 +2348,7 @@
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>phagocytic vesicle</t>
+          <t>mitochondrial proton-transporting ATP synthase, catalytic core</t>
         </is>
       </c>
       <c r="B193" t="n">
@@ -2358,7 +2358,7 @@
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>mitochondrial proton-transporting ATP synthase, catalytic core</t>
+          <t>phagocytic vesicle</t>
         </is>
       </c>
       <c r="B194" t="n">
@@ -2368,7 +2368,7 @@
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>prospore membrane leading edge</t>
+          <t>mitochondrial respirasome</t>
         </is>
       </c>
       <c r="B195" t="n">
@@ -2388,7 +2388,7 @@
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>cytosolic ribosome</t>
+          <t>signal recognition particle</t>
         </is>
       </c>
       <c r="B197" t="n">
@@ -2398,7 +2398,7 @@
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>cytoplasmic side of plasma membrane</t>
+          <t>extrinsic component of vacuolar membrane</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -2408,7 +2408,7 @@
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>vacuolar lumen</t>
+          <t>cell wall-bounded periplasmic space</t>
         </is>
       </c>
       <c r="B199" t="n">
@@ -2418,7 +2418,7 @@
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>cell wall-bounded periplasmic space</t>
+          <t>extrinsic component of plasma membrane</t>
         </is>
       </c>
       <c r="B200" t="n">
@@ -2428,7 +2428,7 @@
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>extrinsic component of vacuolar membrane</t>
+          <t>proteasome regulatory particle</t>
         </is>
       </c>
       <c r="B201" t="n">
@@ -2438,7 +2438,7 @@
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>proteasome regulatory particle</t>
+          <t>spore wall</t>
         </is>
       </c>
       <c r="B202" t="n">
@@ -2448,7 +2448,7 @@
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>spore wall</t>
+          <t>cellular bud neck septin collar</t>
         </is>
       </c>
       <c r="B203" t="n">
@@ -2458,7 +2458,7 @@
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>extrinsic component of plasma membrane</t>
+          <t>cytoplasmic side of plasma membrane</t>
         </is>
       </c>
       <c r="B204" t="n">
@@ -2468,7 +2468,7 @@
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>cellular bud neck septin collar</t>
+          <t>vacuolar lumen</t>
         </is>
       </c>
       <c r="B205" t="n">
@@ -2478,7 +2478,7 @@
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>nuclear outer membrane</t>
+          <t>nucleolar chromatin</t>
         </is>
       </c>
       <c r="B206" t="n">
@@ -2488,7 +2488,7 @@
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>kinetochore microtubule</t>
+          <t>mitochondrial inner boundary membrane</t>
         </is>
       </c>
       <c r="B207" t="n">
@@ -2498,7 +2498,7 @@
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>division septum</t>
+          <t>medial cortex</t>
         </is>
       </c>
       <c r="B208" t="n">
@@ -2508,7 +2508,7 @@
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>mitochondrial chromosome</t>
+          <t>nuclear outer membrane</t>
         </is>
       </c>
       <c r="B209" t="n">
@@ -2518,7 +2518,7 @@
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>mitochondrial proton-transporting ATP synthase, central stalk</t>
+          <t>mating projection base</t>
         </is>
       </c>
       <c r="B210" t="n">
@@ -2528,7 +2528,7 @@
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>mitochondrial inner boundary membrane</t>
+          <t>mitochondrial chromosome</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -2538,7 +2538,7 @@
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>cellular bud neck split septin rings</t>
+          <t>extrinsic component of cytoplasmic side of plasma membrane</t>
         </is>
       </c>
       <c r="B212" t="n">
@@ -2548,7 +2548,7 @@
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>extrinsic component of cytoplasmic side of plasma membrane</t>
+          <t>mitochondrial proton-transporting ATP synthase, central stalk</t>
         </is>
       </c>
       <c r="B213" t="n">
@@ -2558,7 +2558,7 @@
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>medial cortex</t>
+          <t>kinetochore microtubule</t>
         </is>
       </c>
       <c r="B214" t="n">
@@ -2568,7 +2568,7 @@
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>nucleolar chromatin</t>
+          <t>division septum</t>
         </is>
       </c>
       <c r="B215" t="n">
@@ -2578,7 +2578,7 @@
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>mating projection base</t>
+          <t>cellular bud neck split septin rings</t>
         </is>
       </c>
       <c r="B216" t="n">
@@ -2588,7 +2588,7 @@
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>mitochondrial degradosome</t>
+          <t>nuclear envelope lumen</t>
         </is>
       </c>
       <c r="B217" t="n">
@@ -2598,7 +2598,7 @@
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>nuclear matrix</t>
+          <t>mitochondria-associated endoplasmic reticulum membrane</t>
         </is>
       </c>
       <c r="B218" t="n">
@@ -2628,7 +2628,7 @@
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>anchored component of plasma membrane</t>
+          <t>mitochondrial degradosome</t>
         </is>
       </c>
       <c r="B221" t="n">
@@ -2638,7 +2638,7 @@
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>mitochondria-associated endoplasmic reticulum membrane</t>
+          <t>nuclear matrix</t>
         </is>
       </c>
       <c r="B222" t="n">
@@ -2648,7 +2648,7 @@
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>nuclear envelope lumen</t>
+          <t>anchored component of plasma membrane</t>
         </is>
       </c>
       <c r="B223" t="n">
@@ -2658,7 +2658,7 @@
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>cell cortex of growing cell tip</t>
+          <t>mating-type region heterochromatin</t>
         </is>
       </c>
       <c r="B224" t="n">
@@ -2668,7 +2668,7 @@
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>septin filament array</t>
+          <t>mitotic actomyosin contractile ring</t>
         </is>
       </c>
       <c r="B225" t="n">
@@ -2678,7 +2678,7 @@
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>extrinsic component of intraperoxisomal membrane</t>
+          <t>extrinsic component of mitochondrial outer membrane</t>
         </is>
       </c>
       <c r="B226" t="n">
@@ -2688,7 +2688,7 @@
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>nucleoid</t>
+          <t>trans-Golgi network transport vesicle</t>
         </is>
       </c>
       <c r="B227" t="n">
@@ -2698,7 +2698,7 @@
     <row r="228">
       <c r="A228" s="1" t="inlineStr">
         <is>
-          <t>mating-type region heterochromatin</t>
+          <t>eisosome filament</t>
         </is>
       </c>
       <c r="B228" t="n">
@@ -2708,7 +2708,7 @@
     <row r="229">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>integral component of nuclear inner membrane</t>
+          <t>septin filament array</t>
         </is>
       </c>
       <c r="B229" t="n">
@@ -2718,7 +2718,7 @@
     <row r="230">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>mitochondrial crista</t>
+          <t>integral component of nuclear outer membrane</t>
         </is>
       </c>
       <c r="B230" t="n">
@@ -2728,7 +2728,7 @@
     <row r="231">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>tubular endosome</t>
+          <t>mating projection tip membrane</t>
         </is>
       </c>
       <c r="B231" t="n">
@@ -2738,7 +2738,7 @@
     <row r="232">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>proton-transporting V-type ATPase, V1 domain</t>
+          <t>matrix side of mitochondrial inner membrane</t>
         </is>
       </c>
       <c r="B232" t="n">
@@ -2748,7 +2748,7 @@
     <row r="233">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>RNA polymerase II, holoenzyme</t>
+          <t>integral component of nuclear inner membrane</t>
         </is>
       </c>
       <c r="B233" t="n">
@@ -2758,7 +2758,7 @@
     <row r="234">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>integral component of nuclear outer membrane</t>
+          <t>tubular endosome</t>
         </is>
       </c>
       <c r="B234" t="n">
@@ -2768,7 +2768,7 @@
     <row r="235">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>eisosome filament</t>
+          <t>cell cortex of growing cell tip</t>
         </is>
       </c>
       <c r="B235" t="n">
@@ -2778,7 +2778,7 @@
     <row r="236">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>mating projection tip membrane</t>
+          <t>CENP-A containing nucleosome</t>
         </is>
       </c>
       <c r="B236" t="n">
@@ -2788,7 +2788,7 @@
     <row r="237">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>mitotic actomyosin contractile ring</t>
+          <t>mitochondrial crista</t>
         </is>
       </c>
       <c r="B237" t="n">
@@ -2798,7 +2798,7 @@
     <row r="238">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>matrix side of mitochondrial inner membrane</t>
+          <t>extrinsic component of intraperoxisomal membrane</t>
         </is>
       </c>
       <c r="B238" t="n">
@@ -2808,7 +2808,7 @@
     <row r="239">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>extrinsic component of mitochondrial outer membrane</t>
+          <t>RNA polymerase II, holoenzyme</t>
         </is>
       </c>
       <c r="B239" t="n">
@@ -2818,7 +2818,7 @@
     <row r="240">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>trans-Golgi network transport vesicle</t>
+          <t>proton-transporting V-type ATPase, V1 domain</t>
         </is>
       </c>
       <c r="B240" t="n">
@@ -2828,7 +2828,7 @@
     <row r="241">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>CENP-A containing nucleosome</t>
+          <t>nucleoid</t>
         </is>
       </c>
       <c r="B241" t="n">
@@ -2838,7 +2838,7 @@
     <row r="242">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>multivesicular body membrane</t>
+          <t>Golgi-associated vesicle</t>
         </is>
       </c>
       <c r="B242" t="n">
@@ -2848,7 +2848,7 @@
     <row r="243">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>intrinsic component of the cytoplasmic side of the plasma membrane</t>
+          <t>intrinsic component of endoplasmic reticulum membrane</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -2858,7 +2858,7 @@
     <row r="244">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>Golgi to plasma membrane transport vesicle</t>
+          <t>nuclear speck</t>
         </is>
       </c>
       <c r="B244" t="n">
@@ -2868,7 +2868,7 @@
     <row r="245">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>transport vesicle membrane</t>
+          <t>intrinsic component of the cytoplasmic side of the plasma membrane</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -2878,7 +2878,7 @@
     <row r="246">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>cis-Golgi network membrane</t>
+          <t>cytoplasmic side of membrane</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -2888,7 +2888,7 @@
     <row r="247">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>integral component of cytoplasmic side of endoplasmic reticulum membrane</t>
+          <t>anchored component of the cytoplasmic side of the plasma membrane</t>
         </is>
       </c>
       <c r="B247" t="n">
@@ -2898,7 +2898,7 @@
     <row r="248">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>replisome</t>
+          <t>multivesicular body membrane</t>
         </is>
       </c>
       <c r="B248" t="n">
@@ -2908,7 +2908,7 @@
     <row r="249">
       <c r="A249" s="1" t="inlineStr">
         <is>
-          <t>Golgi-associated vesicle</t>
+          <t>Golgi cisterna</t>
         </is>
       </c>
       <c r="B249" t="n">
@@ -2918,7 +2918,7 @@
     <row r="250">
       <c r="A250" s="1" t="inlineStr">
         <is>
-          <t>ascospore-type prospore</t>
+          <t>clathrin coat of trans-Golgi network vesicle</t>
         </is>
       </c>
       <c r="B250" t="n">
@@ -2928,7 +2928,7 @@
     <row r="251">
       <c r="A251" s="1" t="inlineStr">
         <is>
-          <t>astral microtubule</t>
+          <t>integral component of cytoplasmic side of endoplasmic reticulum membrane</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -2938,7 +2938,7 @@
     <row r="252">
       <c r="A252" s="1" t="inlineStr">
         <is>
-          <t>Golgi cisterna</t>
+          <t>astral microtubule</t>
         </is>
       </c>
       <c r="B252" t="n">
@@ -2958,7 +2958,7 @@
     <row r="254">
       <c r="A254" s="1" t="inlineStr">
         <is>
-          <t>clathrin coat of trans-Golgi network vesicle</t>
+          <t>mitotic actomyosin contractile ring, proximal layer</t>
         </is>
       </c>
       <c r="B254" t="n">
@@ -2968,7 +2968,7 @@
     <row r="255">
       <c r="A255" s="1" t="inlineStr">
         <is>
-          <t>cytoplasmic side of membrane</t>
+          <t>transport vesicle membrane</t>
         </is>
       </c>
       <c r="B255" t="n">
@@ -2978,7 +2978,7 @@
     <row r="256">
       <c r="A256" s="1" t="inlineStr">
         <is>
-          <t>anchored component of the cytoplasmic side of the plasma membrane</t>
+          <t>cis-Golgi network membrane</t>
         </is>
       </c>
       <c r="B256" t="n">
@@ -2988,7 +2988,7 @@
     <row r="257">
       <c r="A257" s="1" t="inlineStr">
         <is>
-          <t>nuclear speck</t>
+          <t>ascospore-type prospore</t>
         </is>
       </c>
       <c r="B257" t="n">
@@ -2998,7 +2998,7 @@
     <row r="258">
       <c r="A258" s="1" t="inlineStr">
         <is>
-          <t>intrinsic component of endoplasmic reticulum membrane</t>
+          <t>replisome</t>
         </is>
       </c>
       <c r="B258" t="n">
@@ -3008,7 +3008,7 @@
     <row r="259">
       <c r="A259" s="1" t="inlineStr">
         <is>
-          <t>mitotic actomyosin contractile ring, proximal layer</t>
+          <t>Golgi to plasma membrane transport vesicle</t>
         </is>
       </c>
       <c r="B259" t="n">
@@ -3018,7 +3018,7 @@
     <row r="260">
       <c r="A260" s="1" t="inlineStr">
         <is>
-          <t>replication compartment</t>
+          <t>integral component of lumenal side of endoplasmic reticulum membrane</t>
         </is>
       </c>
       <c r="B260" t="n">
@@ -3028,7 +3028,7 @@
     <row r="261">
       <c r="A261" s="1" t="inlineStr">
         <is>
-          <t>polar microtubule</t>
+          <t>preribosome</t>
         </is>
       </c>
       <c r="B261" t="n">
@@ -3038,7 +3038,7 @@
     <row r="262">
       <c r="A262" s="1" t="inlineStr">
         <is>
-          <t>Golgi cisterna membrane</t>
+          <t>cortical microtubule plus-end</t>
         </is>
       </c>
       <c r="B262" t="n">
@@ -3048,7 +3048,7 @@
     <row r="263">
       <c r="A263" s="1" t="inlineStr">
         <is>
-          <t>preribosome</t>
+          <t>lateral element</t>
         </is>
       </c>
       <c r="B263" t="n">
@@ -3058,7 +3058,7 @@
     <row r="264">
       <c r="A264" s="1" t="inlineStr">
         <is>
-          <t>plasma membrane of growing cell tip</t>
+          <t>chromosome, centromeric core domain</t>
         </is>
       </c>
       <c r="B264" t="n">
@@ -3068,7 +3068,7 @@
     <row r="265">
       <c r="A265" s="1" t="inlineStr">
         <is>
-          <t>autophagosome membrane</t>
+          <t>intrinsic component of vacuolar membrane</t>
         </is>
       </c>
       <c r="B265" t="n">
@@ -3078,7 +3078,7 @@
     <row r="266">
       <c r="A266" s="1" t="inlineStr">
         <is>
-          <t>intrinsic component of vacuolar membrane</t>
+          <t>cellular birth scar</t>
         </is>
       </c>
       <c r="B266" t="n">
@@ -3088,7 +3088,7 @@
     <row r="267">
       <c r="A267" s="1" t="inlineStr">
         <is>
-          <t>P granule</t>
+          <t>replication compartment</t>
         </is>
       </c>
       <c r="B267" t="n">
@@ -3098,7 +3098,7 @@
     <row r="268">
       <c r="A268" s="1" t="inlineStr">
         <is>
-          <t>cytoplasmic side of mitochondrial outer membrane</t>
+          <t>mating projection membrane</t>
         </is>
       </c>
       <c r="B268" t="n">
@@ -3108,7 +3108,7 @@
     <row r="269">
       <c r="A269" s="1" t="inlineStr">
         <is>
-          <t>cellular birth scar</t>
+          <t>cytoplasmic side of mitochondrial outer membrane</t>
         </is>
       </c>
       <c r="B269" t="n">
@@ -3118,7 +3118,7 @@
     <row r="270">
       <c r="A270" s="1" t="inlineStr">
         <is>
-          <t>mating projection membrane</t>
+          <t>heterochromatin</t>
         </is>
       </c>
       <c r="B270" t="n">
@@ -3128,7 +3128,7 @@
     <row r="271">
       <c r="A271" s="1" t="inlineStr">
         <is>
-          <t>heterochromatin</t>
+          <t>P granule</t>
         </is>
       </c>
       <c r="B271" t="n">
@@ -3138,7 +3138,7 @@
     <row r="272">
       <c r="A272" s="1" t="inlineStr">
         <is>
-          <t>nuclear pore linkers</t>
+          <t>lytic vacuole</t>
         </is>
       </c>
       <c r="B272" t="n">
@@ -3148,7 +3148,7 @@
     <row r="273">
       <c r="A273" s="1" t="inlineStr">
         <is>
-          <t>outer kinetochore</t>
+          <t>Golgi cisterna membrane</t>
         </is>
       </c>
       <c r="B273" t="n">
@@ -3158,7 +3158,7 @@
     <row r="274">
       <c r="A274" s="1" t="inlineStr">
         <is>
-          <t>2-micrometer circle DNA</t>
+          <t>polar microtubule</t>
         </is>
       </c>
       <c r="B274" t="n">
@@ -3168,7 +3168,7 @@
     <row r="275">
       <c r="A275" s="1" t="inlineStr">
         <is>
-          <t>cortical microtubule plus-end</t>
+          <t>chitosome</t>
         </is>
       </c>
       <c r="B275" t="n">
@@ -3178,7 +3178,7 @@
     <row r="276">
       <c r="A276" s="1" t="inlineStr">
         <is>
-          <t>lytic vacuole</t>
+          <t>nuclear body</t>
         </is>
       </c>
       <c r="B276" t="n">
@@ -3188,7 +3188,7 @@
     <row r="277">
       <c r="A277" s="1" t="inlineStr">
         <is>
-          <t>nucleolar preribosome</t>
+          <t>extracellular matrix</t>
         </is>
       </c>
       <c r="B277" t="n">
@@ -3198,7 +3198,7 @@
     <row r="278">
       <c r="A278" s="1" t="inlineStr">
         <is>
-          <t>chromosome, centromeric core domain</t>
+          <t>integral component of endosome membrane</t>
         </is>
       </c>
       <c r="B278" t="n">
@@ -3208,7 +3208,7 @@
     <row r="279">
       <c r="A279" s="1" t="inlineStr">
         <is>
-          <t>nuclear body</t>
+          <t>nuclear pore linkers</t>
         </is>
       </c>
       <c r="B279" t="n">
@@ -3218,7 +3218,7 @@
     <row r="280">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>integral component of lumenal side of endoplasmic reticulum membrane</t>
+          <t>autophagosome membrane</t>
         </is>
       </c>
       <c r="B280" t="n">
@@ -3228,7 +3228,7 @@
     <row r="281">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>integral component of endosome membrane</t>
+          <t>integral component of organelle membrane</t>
         </is>
       </c>
       <c r="B281" t="n">
@@ -3238,7 +3238,7 @@
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>nuclear inclusion body</t>
+          <t>2-micrometer circle DNA</t>
         </is>
       </c>
       <c r="B282" t="n">
@@ -3248,7 +3248,7 @@
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>lateral element</t>
+          <t>outer membrane</t>
         </is>
       </c>
       <c r="B283" t="n">
@@ -3258,7 +3258,7 @@
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>extracellular matrix</t>
+          <t>outer kinetochore</t>
         </is>
       </c>
       <c r="B284" t="n">
@@ -3268,7 +3268,7 @@
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>integral component of organelle membrane</t>
+          <t>nuclear inclusion body</t>
         </is>
       </c>
       <c r="B285" t="n">
@@ -3278,7 +3278,7 @@
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>chitosome</t>
+          <t>nucleolar preribosome</t>
         </is>
       </c>
       <c r="B286" t="n">
@@ -3298,7 +3298,7 @@
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>outer membrane</t>
+          <t>plasma membrane of growing cell tip</t>
         </is>
       </c>
       <c r="B288" t="n">
@@ -3308,7 +3308,7 @@
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>nuclear replisome</t>
+          <t>integral component of vacuolar membrane</t>
         </is>
       </c>
       <c r="B289" t="n">
@@ -3318,7 +3318,7 @@
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>DNA replication termination region</t>
+          <t>retrotransposon nucleocapsid</t>
         </is>
       </c>
       <c r="B290" t="n">
@@ -3328,7 +3328,7 @@
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>host cell viral assembly compartment</t>
+          <t>intermediate filament</t>
         </is>
       </c>
       <c r="B291" t="n">
@@ -3338,7 +3338,7 @@
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>perinuclear endoplasmic reticulum membrane</t>
+          <t>endoplasmic reticulum-Golgi intermediate compartment membrane</t>
         </is>
       </c>
       <c r="B292" t="n">
@@ -3348,7 +3348,7 @@
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>eisosome membrane domain/MCC</t>
+          <t>endoplasmic reticulum quality control compartment</t>
         </is>
       </c>
       <c r="B293" t="n">
@@ -3358,7 +3358,7 @@
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>extrinsic component of matrix side of mitochondrial inner membrane</t>
+          <t>perinuclear endoplasmic reticulum membrane</t>
         </is>
       </c>
       <c r="B294" t="n">
@@ -3368,7 +3368,7 @@
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>Cvt vesicle membrane</t>
+          <t>trans-Golgi network transport vesicle membrane</t>
         </is>
       </c>
       <c r="B295" t="n">
@@ -3378,7 +3378,7 @@
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>primary cell septum</t>
+          <t>eisosome membrane domain/MCC</t>
         </is>
       </c>
       <c r="B296" t="n">
@@ -3388,7 +3388,7 @@
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>intermediate filament</t>
+          <t>extrinsic component of matrix side of mitochondrial inner membrane</t>
         </is>
       </c>
       <c r="B297" t="n">
@@ -3398,7 +3398,7 @@
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>prespliceosome</t>
+          <t>cytoplasmic ribonucleoprotein granule</t>
         </is>
       </c>
       <c r="B298" t="n">
@@ -3408,7 +3408,7 @@
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>extrinsic component of nuclear outer membrane</t>
+          <t>cytoplasmic side of endosome membrane</t>
         </is>
       </c>
       <c r="B299" t="n">
@@ -3418,7 +3418,7 @@
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>retrotransposon nucleocapsid</t>
+          <t>ascus lipid droplet</t>
         </is>
       </c>
       <c r="B300" t="n">
@@ -3428,7 +3428,7 @@
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>organelle membrane</t>
+          <t>prespliceosome</t>
         </is>
       </c>
       <c r="B301" t="n">
@@ -3448,7 +3448,7 @@
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>endoplasmic reticulum quality control compartment</t>
+          <t>host cell viral assembly compartment</t>
         </is>
       </c>
       <c r="B303" t="n">
@@ -3458,7 +3458,7 @@
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>endoplasmic reticulum-Golgi intermediate compartment membrane</t>
+          <t>endocytic patch</t>
         </is>
       </c>
       <c r="B304" t="n">
@@ -3468,7 +3468,7 @@
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>prospore septin filament array</t>
+          <t>ruffle membrane</t>
         </is>
       </c>
       <c r="B305" t="n">
@@ -3478,7 +3478,7 @@
     <row r="306">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>cell wall</t>
+          <t>organelle membrane contact site</t>
         </is>
       </c>
       <c r="B306" t="n">
@@ -3488,7 +3488,7 @@
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>integral component of vacuolar membrane</t>
+          <t>organelle membrane</t>
         </is>
       </c>
       <c r="B307" t="n">
@@ -3498,7 +3498,7 @@
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>cytoplasmic side of endosome membrane</t>
+          <t>nuclear replisome</t>
         </is>
       </c>
       <c r="B308" t="n">
@@ -3508,7 +3508,7 @@
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>endocytic patch</t>
+          <t>extrinsic component of nuclear outer membrane</t>
         </is>
       </c>
       <c r="B309" t="n">
@@ -3518,7 +3518,7 @@
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>trans-Golgi network transport vesicle membrane</t>
+          <t>DNA replication termination region</t>
         </is>
       </c>
       <c r="B310" t="n">
@@ -3528,7 +3528,7 @@
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>transverse filament</t>
+          <t>prospore septin filament array</t>
         </is>
       </c>
       <c r="B311" t="n">
@@ -3538,7 +3538,7 @@
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>cytoplasmic ribonucleoprotein granule</t>
+          <t>transverse filament</t>
         </is>
       </c>
       <c r="B312" t="n">
@@ -3548,7 +3548,7 @@
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>ascus lipid droplet</t>
+          <t>Cvt vesicle membrane</t>
         </is>
       </c>
       <c r="B313" t="n">
@@ -3558,7 +3558,7 @@
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>ruffle membrane</t>
+          <t>primary cell septum</t>
         </is>
       </c>
       <c r="B314" t="n">
@@ -3568,7 +3568,7 @@
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>organelle membrane contact site</t>
+          <t>cell wall</t>
         </is>
       </c>
       <c r="B315" t="n">

</xml_diff>

<commit_message>
fix: optimize the module
</commit_message>
<xml_diff>
--- a/data/all_component_analysis.xlsx
+++ b/data/all_component_analysis.xlsx
@@ -838,7 +838,7 @@
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>P-body</t>
+          <t>kinetochore</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -848,7 +848,7 @@
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>kinetochore</t>
+          <t>P-body</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1348,7 +1348,7 @@
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>clathrin-coated vesicle</t>
+          <t>membrane raft</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -1358,7 +1358,7 @@
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>membrane raft</t>
+          <t>clathrin-coated vesicle</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -1438,7 +1438,7 @@
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>endoplasmic reticulum exit site</t>
+          <t>integral component of peroxisomal membrane</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -1448,7 +1448,7 @@
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
         <is>
-          <t>cytoplasmic microtubule</t>
+          <t>endoplasmic reticulum exit site</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -1458,7 +1458,7 @@
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t>integral component of peroxisomal membrane</t>
+          <t>cytoplasmic microtubule</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -1498,7 +1498,7 @@
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>cis-Golgi network</t>
+          <t>signal recognition particle, endoplasmic reticulum targeting</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -1508,7 +1508,7 @@
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>signal recognition particle, endoplasmic reticulum targeting</t>
+          <t>cis-Golgi network</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -1578,7 +1578,7 @@
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>replication fork</t>
+          <t>nucleosome</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -1598,7 +1598,7 @@
     <row r="118">
       <c r="A118" s="1" t="inlineStr">
         <is>
-          <t>nucleosome</t>
+          <t>ER to Golgi transport vesicle membrane</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -1608,7 +1608,7 @@
     <row r="119">
       <c r="A119" s="1" t="inlineStr">
         <is>
-          <t>ER to Golgi transport vesicle membrane</t>
+          <t>replication fork</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -1668,7 +1668,7 @@
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>autophagosome</t>
+          <t>cellular bud neck contractile ring</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -1688,7 +1688,7 @@
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>cellular bud neck contractile ring</t>
+          <t>autophagosome</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -1698,7 +1698,7 @@
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>COP9 signalosome</t>
+          <t>condensed chromosome, centromeric region</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -1708,7 +1708,7 @@
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>condensed chromosome, centromeric region</t>
+          <t>COP9 signalosome</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -1718,7 +1718,7 @@
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>multivesicular body</t>
+          <t>fungal-type vacuole lumen</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -1728,7 +1728,7 @@
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>fungal-type vacuole lumen</t>
+          <t>multivesicular body</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -1738,7 +1738,7 @@
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>ascospore wall</t>
+          <t>cellular bud neck septin ring</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -1748,7 +1748,7 @@
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>late endosome membrane</t>
+          <t>ascospore wall</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -1758,7 +1758,7 @@
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>cellular bud neck septin ring</t>
+          <t>late endosome membrane</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -1768,7 +1768,7 @@
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>nuclear chromosome</t>
+          <t>microtubule organizing center</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -1798,7 +1798,7 @@
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>microtubule organizing center</t>
+          <t>nuclear chromosome</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -1868,7 +1868,7 @@
     <row r="145">
       <c r="A145" s="1" t="inlineStr">
         <is>
-          <t>nucleus-vacuole junction</t>
+          <t>integral component of fungal-type vacuolar membrane</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -1878,7 +1878,7 @@
     <row r="146">
       <c r="A146" s="1" t="inlineStr">
         <is>
-          <t>integral component of fungal-type vacuolar membrane</t>
+          <t>nucleus-vacuole junction</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -1888,7 +1888,7 @@
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>nuclear pore cytoplasmic filaments</t>
+          <t>integral component of mitochondrial membrane</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -1898,7 +1898,7 @@
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>vacuolar proton-transporting V-type ATPase, V1 domain</t>
+          <t>endocytic vesicle</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -1908,7 +1908,7 @@
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>nuclear pore transmembrane ring</t>
+          <t>cell cortex of cell tip</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -1918,7 +1918,7 @@
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>cell cortex of cell tip</t>
+          <t>nuclear pore cytoplasmic filaments</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -1928,7 +1928,7 @@
     <row r="151">
       <c r="A151" s="1" t="inlineStr">
         <is>
-          <t>integral component of mitochondrial membrane</t>
+          <t>nuclear pore transmembrane ring</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -1938,7 +1938,7 @@
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>endocytic vesicle</t>
+          <t>vacuolar proton-transporting V-type ATPase, V1 domain</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -1958,7 +1958,7 @@
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>transcriptionally active chromatin</t>
+          <t>cytoplasmic vesicle membrane</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -1968,7 +1968,7 @@
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>cytoplasmic vesicle membrane</t>
+          <t>transcriptionally active chromatin</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -1988,7 +1988,7 @@
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>CHRAC</t>
+          <t>vacuolar proton-transporting V-type ATPase, V0 domain</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -1998,7 +1998,7 @@
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>vacuolar proton-transporting V-type ATPase, V0 domain</t>
+          <t>CHRAC</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -2008,7 +2008,7 @@
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>vacuole-mitochondrion membrane contact site</t>
+          <t>nuclear pore nuclear basket</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -2028,7 +2028,7 @@
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>nuclear pore nuclear basket</t>
+          <t>nuclear pore inner ring</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -2038,7 +2038,7 @@
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>nuclear pore inner ring</t>
+          <t>COPI-coated vesicle</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -2048,7 +2048,7 @@
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>COPI-coated vesicle</t>
+          <t>vacuole-mitochondrion membrane contact site</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -2058,7 +2058,7 @@
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>extrinsic component of fungal-type vacuolar membrane</t>
+          <t>Golgi stack</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -2068,7 +2068,7 @@
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>mitochondrial ribosome</t>
+          <t>extrinsic component of fungal-type vacuolar membrane</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -2078,7 +2078,7 @@
     <row r="166">
       <c r="A166" s="1" t="inlineStr">
         <is>
-          <t>Golgi stack</t>
+          <t>mitochondrial ribosome</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -2098,7 +2098,7 @@
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>transport vesicle</t>
+          <t>extrinsic component of endoplasmic reticulum membrane</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -2108,7 +2108,7 @@
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>extrinsic component of endoplasmic reticulum membrane</t>
+          <t>transport vesicle</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -2128,7 +2128,7 @@
     <row r="171">
       <c r="A171" s="1" t="inlineStr">
         <is>
-          <t>rDNA heterochromatin</t>
+          <t>Golgi medial cisterna</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -2138,7 +2138,7 @@
     <row r="172">
       <c r="A172" s="1" t="inlineStr">
         <is>
-          <t>Golgi medial cisterna</t>
+          <t>rDNA heterochromatin</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -2158,7 +2158,7 @@
     <row r="174">
       <c r="A174" s="1" t="inlineStr">
         <is>
-          <t>equatorial microtubule organizing center</t>
+          <t>cellular bud membrane</t>
         </is>
       </c>
       <c r="B174" t="n">
@@ -2168,7 +2168,7 @@
     <row r="175">
       <c r="A175" s="1" t="inlineStr">
         <is>
-          <t>cellular bud membrane</t>
+          <t>equatorial microtubule organizing center</t>
         </is>
       </c>
       <c r="B175" t="n">
@@ -2178,7 +2178,7 @@
     <row r="176">
       <c r="A176" s="1" t="inlineStr">
         <is>
-          <t>mating projection</t>
+          <t>endoplasmic reticulum tubular network</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -2188,7 +2188,7 @@
     <row r="177">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>intrinsic component of mitochondrial inner membrane</t>
+          <t>mating projection</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -2198,7 +2198,7 @@
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>endoplasmic reticulum tubular network</t>
+          <t>early endosome membrane</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -2208,7 +2208,7 @@
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>phagophore</t>
+          <t>growing cell tip</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -2218,7 +2218,7 @@
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>vacuole-isolation membrane contact site</t>
+          <t>mitochondrial crista junction</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -2228,7 +2228,7 @@
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>growing cell tip</t>
+          <t>Golgi cis cisterna</t>
         </is>
       </c>
       <c r="B181" t="n">
@@ -2238,7 +2238,7 @@
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>mitochondrial crista junction</t>
+          <t>Golgi trans cisterna</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -2258,7 +2258,7 @@
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>Golgi cis cisterna</t>
+          <t>clathrin-coated vesicle membrane</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -2268,7 +2268,7 @@
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>clathrin-coated vesicle membrane</t>
+          <t>phagophore</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -2278,7 +2278,7 @@
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>Golgi trans cisterna</t>
+          <t>vacuole-isolation membrane contact site</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -2288,7 +2288,7 @@
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>early endosome membrane</t>
+          <t>intrinsic component of mitochondrial inner membrane</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -2308,7 +2308,7 @@
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>polarisome</t>
+          <t>cytosolic ribosome</t>
         </is>
       </c>
       <c r="B189" t="n">
@@ -2318,7 +2318,7 @@
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>mitochondrial respirasome</t>
+          <t>phagocytic vesicle</t>
         </is>
       </c>
       <c r="B190" t="n">
@@ -2328,7 +2328,7 @@
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>cytosolic ribosome</t>
+          <t>nuclear microtubule</t>
         </is>
       </c>
       <c r="B191" t="n">
@@ -2338,7 +2338,7 @@
     <row r="192">
       <c r="A192" s="1" t="inlineStr">
         <is>
-          <t>mitochondrial proton-transporting ATP synthase, catalytic core</t>
+          <t>polarisome</t>
         </is>
       </c>
       <c r="B192" t="n">
@@ -2348,7 +2348,7 @@
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>nuclear microtubule</t>
+          <t>mitochondrial proton-transporting ATP synthase, catalytic core</t>
         </is>
       </c>
       <c r="B193" t="n">
@@ -2368,7 +2368,7 @@
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>condensed chromosome</t>
+          <t>mitochondrial respirasome</t>
         </is>
       </c>
       <c r="B195" t="n">
@@ -2378,7 +2378,7 @@
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>signal recognition particle</t>
+          <t>condensed chromosome</t>
         </is>
       </c>
       <c r="B196" t="n">
@@ -2388,7 +2388,7 @@
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>phagocytic vesicle</t>
+          <t>signal recognition particle</t>
         </is>
       </c>
       <c r="B197" t="n">
@@ -2398,7 +2398,7 @@
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>spore wall</t>
+          <t>cell wall-bounded periplasmic space</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -2408,7 +2408,7 @@
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>vacuolar lumen</t>
+          <t>extrinsic component of vacuolar membrane</t>
         </is>
       </c>
       <c r="B199" t="n">
@@ -2418,7 +2418,7 @@
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>cytoplasmic side of plasma membrane</t>
+          <t>cellular bud neck septin collar</t>
         </is>
       </c>
       <c r="B200" t="n">
@@ -2428,7 +2428,7 @@
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>proteasome regulatory particle</t>
+          <t>vacuolar lumen</t>
         </is>
       </c>
       <c r="B201" t="n">
@@ -2438,7 +2438,7 @@
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>cell wall-bounded periplasmic space</t>
+          <t>proteasome regulatory particle</t>
         </is>
       </c>
       <c r="B202" t="n">
@@ -2448,7 +2448,7 @@
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>extrinsic component of vacuolar membrane</t>
+          <t>spore wall</t>
         </is>
       </c>
       <c r="B203" t="n">
@@ -2458,7 +2458,7 @@
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>extrinsic component of plasma membrane</t>
+          <t>cytoplasmic side of plasma membrane</t>
         </is>
       </c>
       <c r="B204" t="n">
@@ -2468,7 +2468,7 @@
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>cellular bud neck septin collar</t>
+          <t>extrinsic component of plasma membrane</t>
         </is>
       </c>
       <c r="B205" t="n">
@@ -2478,7 +2478,7 @@
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>kinetochore microtubule</t>
+          <t>nuclear outer membrane</t>
         </is>
       </c>
       <c r="B206" t="n">
@@ -2488,7 +2488,7 @@
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>mating projection base</t>
+          <t>mitochondrial chromosome</t>
         </is>
       </c>
       <c r="B207" t="n">
@@ -2498,7 +2498,7 @@
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>mitochondrial proton-transporting ATP synthase, central stalk</t>
+          <t>mitochondrial inner boundary membrane</t>
         </is>
       </c>
       <c r="B208" t="n">
@@ -2508,7 +2508,7 @@
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>nucleolar chromatin</t>
+          <t>mating projection base</t>
         </is>
       </c>
       <c r="B209" t="n">
@@ -2528,7 +2528,7 @@
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>mitochondrial chromosome</t>
+          <t>division septum</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -2538,7 +2538,7 @@
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>medial cortex</t>
+          <t>nucleolar chromatin</t>
         </is>
       </c>
       <c r="B212" t="n">
@@ -2548,7 +2548,7 @@
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>nuclear outer membrane</t>
+          <t>medial cortex</t>
         </is>
       </c>
       <c r="B213" t="n">
@@ -2558,7 +2558,7 @@
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>division septum</t>
+          <t>kinetochore microtubule</t>
         </is>
       </c>
       <c r="B214" t="n">
@@ -2568,7 +2568,7 @@
     <row r="215">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>mitochondrial inner boundary membrane</t>
+          <t>cellular bud neck split septin rings</t>
         </is>
       </c>
       <c r="B215" t="n">
@@ -2578,7 +2578,7 @@
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>cellular bud neck split septin rings</t>
+          <t>mitochondrial proton-transporting ATP synthase, central stalk</t>
         </is>
       </c>
       <c r="B216" t="n">
@@ -2588,7 +2588,7 @@
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>anchored component of plasma membrane</t>
+          <t>nuclear matrix</t>
         </is>
       </c>
       <c r="B217" t="n">
@@ -2598,7 +2598,7 @@
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>mitochondria-associated endoplasmic reticulum membrane</t>
+          <t>anchored component of plasma membrane</t>
         </is>
       </c>
       <c r="B218" t="n">
@@ -2608,7 +2608,7 @@
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>mitochondrial degradosome</t>
+          <t>mitochondria-associated endoplasmic reticulum membrane</t>
         </is>
       </c>
       <c r="B219" t="n">
@@ -2618,7 +2618,7 @@
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>nuclear matrix</t>
+          <t>mitochondrial degradosome</t>
         </is>
       </c>
       <c r="B220" t="n">
@@ -2638,7 +2638,7 @@
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>polysomal ribosome</t>
+          <t>membrane-bounded organelle</t>
         </is>
       </c>
       <c r="B222" t="n">
@@ -2648,7 +2648,7 @@
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>membrane-bounded organelle</t>
+          <t>polysomal ribosome</t>
         </is>
       </c>
       <c r="B223" t="n">
@@ -2658,7 +2658,7 @@
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>mating projection tip membrane</t>
+          <t>RNA polymerase II, holoenzyme</t>
         </is>
       </c>
       <c r="B224" t="n">
@@ -2668,7 +2668,7 @@
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>matrix side of mitochondrial inner membrane</t>
+          <t>mitotic actomyosin contractile ring</t>
         </is>
       </c>
       <c r="B225" t="n">
@@ -2678,7 +2678,7 @@
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>proton-transporting V-type ATPase, V1 domain</t>
+          <t>eisosome filament</t>
         </is>
       </c>
       <c r="B226" t="n">
@@ -2688,7 +2688,7 @@
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>cell cortex of growing cell tip</t>
+          <t>trans-Golgi network transport vesicle</t>
         </is>
       </c>
       <c r="B227" t="n">
@@ -2698,7 +2698,7 @@
     <row r="228">
       <c r="A228" s="1" t="inlineStr">
         <is>
-          <t>mitotic actomyosin contractile ring</t>
+          <t>mitochondrial crista</t>
         </is>
       </c>
       <c r="B228" t="n">
@@ -2708,7 +2708,7 @@
     <row r="229">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>mitochondrial crista</t>
+          <t>matrix side of mitochondrial inner membrane</t>
         </is>
       </c>
       <c r="B229" t="n">
@@ -2718,7 +2718,7 @@
     <row r="230">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>mating-type region heterochromatin</t>
+          <t>integral component of nuclear inner membrane</t>
         </is>
       </c>
       <c r="B230" t="n">
@@ -2728,7 +2728,7 @@
     <row r="231">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>extrinsic component of mitochondrial outer membrane</t>
+          <t>integral component of nuclear outer membrane</t>
         </is>
       </c>
       <c r="B231" t="n">
@@ -2738,7 +2738,7 @@
     <row r="232">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>extrinsic component of intraperoxisomal membrane</t>
+          <t>extrinsic component of mitochondrial outer membrane</t>
         </is>
       </c>
       <c r="B232" t="n">
@@ -2748,7 +2748,7 @@
     <row r="233">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>integral component of nuclear outer membrane</t>
+          <t>septin filament array</t>
         </is>
       </c>
       <c r="B233" t="n">
@@ -2758,7 +2758,7 @@
     <row r="234">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>RNA polymerase II, holoenzyme</t>
+          <t>proton-transporting V-type ATPase, V1 domain</t>
         </is>
       </c>
       <c r="B234" t="n">
@@ -2768,7 +2768,7 @@
     <row r="235">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>eisosome filament</t>
+          <t>tubular endosome</t>
         </is>
       </c>
       <c r="B235" t="n">
@@ -2778,7 +2778,7 @@
     <row r="236">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>CENP-A containing nucleosome</t>
+          <t>mating-type region heterochromatin</t>
         </is>
       </c>
       <c r="B236" t="n">
@@ -2788,7 +2788,7 @@
     <row r="237">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>tubular endosome</t>
+          <t>cell cortex of growing cell tip</t>
         </is>
       </c>
       <c r="B237" t="n">
@@ -2798,7 +2798,7 @@
     <row r="238">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>nucleoid</t>
+          <t>CENP-A containing nucleosome</t>
         </is>
       </c>
       <c r="B238" t="n">
@@ -2808,7 +2808,7 @@
     <row r="239">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>trans-Golgi network transport vesicle</t>
+          <t>extrinsic component of intraperoxisomal membrane</t>
         </is>
       </c>
       <c r="B239" t="n">
@@ -2818,7 +2818,7 @@
     <row r="240">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>integral component of nuclear inner membrane</t>
+          <t>mating projection tip membrane</t>
         </is>
       </c>
       <c r="B240" t="n">
@@ -2828,7 +2828,7 @@
     <row r="241">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>septin filament array</t>
+          <t>nucleoid</t>
         </is>
       </c>
       <c r="B241" t="n">
@@ -2838,7 +2838,7 @@
     <row r="242">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>transport vesicle membrane</t>
+          <t>astral microtubule</t>
         </is>
       </c>
       <c r="B242" t="n">
@@ -2848,7 +2848,7 @@
     <row r="243">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>Golgi-associated vesicle</t>
+          <t>replisome</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -2858,7 +2858,7 @@
     <row r="244">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>Golgi cisterna</t>
+          <t>multivesicular body membrane</t>
         </is>
       </c>
       <c r="B244" t="n">
@@ -2868,7 +2868,7 @@
     <row r="245">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>multivesicular body membrane</t>
+          <t>cis-Golgi network membrane</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -2878,7 +2878,7 @@
     <row r="246">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>nuclear speck</t>
+          <t>Golgi cisterna</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -2888,7 +2888,7 @@
     <row r="247">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>intrinsic component of endoplasmic reticulum membrane</t>
+          <t>transport vesicle membrane</t>
         </is>
       </c>
       <c r="B247" t="n">
@@ -2898,7 +2898,7 @@
     <row r="248">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>integral component of cytoplasmic side of endoplasmic reticulum membrane</t>
+          <t>intrinsic component of endoplasmic reticulum membrane</t>
         </is>
       </c>
       <c r="B248" t="n">
@@ -2908,7 +2908,7 @@
     <row r="249">
       <c r="A249" s="1" t="inlineStr">
         <is>
-          <t>anchored component of the cytoplasmic side of the plasma membrane</t>
+          <t>Golgi to plasma membrane transport vesicle</t>
         </is>
       </c>
       <c r="B249" t="n">
@@ -2918,7 +2918,7 @@
     <row r="250">
       <c r="A250" s="1" t="inlineStr">
         <is>
-          <t>clathrin coat of trans-Golgi network vesicle</t>
+          <t>nuclear speck</t>
         </is>
       </c>
       <c r="B250" t="n">
@@ -2928,7 +2928,7 @@
     <row r="251">
       <c r="A251" s="1" t="inlineStr">
         <is>
-          <t>cytoplasmic side of membrane</t>
+          <t>Golgi-associated vesicle</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -2948,7 +2948,7 @@
     <row r="253">
       <c r="A253" s="1" t="inlineStr">
         <is>
-          <t>replisome</t>
+          <t>anchored component of the cytoplasmic side of the plasma membrane</t>
         </is>
       </c>
       <c r="B253" t="n">
@@ -2958,7 +2958,7 @@
     <row r="254">
       <c r="A254" s="1" t="inlineStr">
         <is>
-          <t>intrinsic component of the cytoplasmic side of the plasma membrane</t>
+          <t>clathrin coat of coated pit</t>
         </is>
       </c>
       <c r="B254" t="n">
@@ -2968,7 +2968,7 @@
     <row r="255">
       <c r="A255" s="1" t="inlineStr">
         <is>
-          <t>Golgi to plasma membrane transport vesicle</t>
+          <t>intrinsic component of the cytoplasmic side of the plasma membrane</t>
         </is>
       </c>
       <c r="B255" t="n">
@@ -2978,7 +2978,7 @@
     <row r="256">
       <c r="A256" s="1" t="inlineStr">
         <is>
-          <t>cis-Golgi network membrane</t>
+          <t>integral component of cytoplasmic side of endoplasmic reticulum membrane</t>
         </is>
       </c>
       <c r="B256" t="n">
@@ -2988,7 +2988,7 @@
     <row r="257">
       <c r="A257" s="1" t="inlineStr">
         <is>
-          <t>clathrin coat of coated pit</t>
+          <t>ascospore-type prospore</t>
         </is>
       </c>
       <c r="B257" t="n">
@@ -2998,7 +2998,7 @@
     <row r="258">
       <c r="A258" s="1" t="inlineStr">
         <is>
-          <t>astral microtubule</t>
+          <t>cytoplasmic side of membrane</t>
         </is>
       </c>
       <c r="B258" t="n">
@@ -3008,7 +3008,7 @@
     <row r="259">
       <c r="A259" s="1" t="inlineStr">
         <is>
-          <t>ascospore-type prospore</t>
+          <t>clathrin coat of trans-Golgi network vesicle</t>
         </is>
       </c>
       <c r="B259" t="n">
@@ -3018,7 +3018,7 @@
     <row r="260">
       <c r="A260" s="1" t="inlineStr">
         <is>
-          <t>outer membrane</t>
+          <t>P granule</t>
         </is>
       </c>
       <c r="B260" t="n">
@@ -3028,7 +3028,7 @@
     <row r="261">
       <c r="A261" s="1" t="inlineStr">
         <is>
-          <t>cellular birth scar</t>
+          <t>integral component of organelle membrane</t>
         </is>
       </c>
       <c r="B261" t="n">
@@ -3038,7 +3038,7 @@
     <row r="262">
       <c r="A262" s="1" t="inlineStr">
         <is>
-          <t>cytoplasmic side of mitochondrial outer membrane</t>
+          <t>cortical microtubule plus-end</t>
         </is>
       </c>
       <c r="B262" t="n">
@@ -3048,7 +3048,7 @@
     <row r="263">
       <c r="A263" s="1" t="inlineStr">
         <is>
-          <t>replication compartment</t>
+          <t>intrinsic component of vacuolar membrane</t>
         </is>
       </c>
       <c r="B263" t="n">
@@ -3058,7 +3058,7 @@
     <row r="264">
       <c r="A264" s="1" t="inlineStr">
         <is>
-          <t>2-micrometer circle DNA</t>
+          <t>cellular birth scar</t>
         </is>
       </c>
       <c r="B264" t="n">
@@ -3068,7 +3068,7 @@
     <row r="265">
       <c r="A265" s="1" t="inlineStr">
         <is>
-          <t>nuclear inclusion body</t>
+          <t>integral component of endosome membrane</t>
         </is>
       </c>
       <c r="B265" t="n">
@@ -3078,7 +3078,7 @@
     <row r="266">
       <c r="A266" s="1" t="inlineStr">
         <is>
-          <t>plasma membrane of growing cell tip</t>
+          <t>replication compartment</t>
         </is>
       </c>
       <c r="B266" t="n">
@@ -3088,7 +3088,7 @@
     <row r="267">
       <c r="A267" s="1" t="inlineStr">
         <is>
-          <t>intrinsic component of vacuolar membrane</t>
+          <t>preribosome</t>
         </is>
       </c>
       <c r="B267" t="n">
@@ -3098,7 +3098,7 @@
     <row r="268">
       <c r="A268" s="1" t="inlineStr">
         <is>
-          <t>outer kinetochore</t>
+          <t>secretory vesicle</t>
         </is>
       </c>
       <c r="B268" t="n">
@@ -3108,7 +3108,7 @@
     <row r="269">
       <c r="A269" s="1" t="inlineStr">
         <is>
-          <t>P granule</t>
+          <t>cytoplasmic side of mitochondrial outer membrane</t>
         </is>
       </c>
       <c r="B269" t="n">
@@ -3118,7 +3118,7 @@
     <row r="270">
       <c r="A270" s="1" t="inlineStr">
         <is>
-          <t>polar microtubule</t>
+          <t>lateral element</t>
         </is>
       </c>
       <c r="B270" t="n">
@@ -3128,7 +3128,7 @@
     <row r="271">
       <c r="A271" s="1" t="inlineStr">
         <is>
-          <t>Golgi cisterna membrane</t>
+          <t>polar microtubule</t>
         </is>
       </c>
       <c r="B271" t="n">
@@ -3138,7 +3138,7 @@
     <row r="272">
       <c r="A272" s="1" t="inlineStr">
         <is>
-          <t>lytic vacuole</t>
+          <t>heterochromatin</t>
         </is>
       </c>
       <c r="B272" t="n">
@@ -3148,7 +3148,7 @@
     <row r="273">
       <c r="A273" s="1" t="inlineStr">
         <is>
-          <t>chromosome, centromeric core domain</t>
+          <t>2-micrometer circle DNA</t>
         </is>
       </c>
       <c r="B273" t="n">
@@ -3158,7 +3158,7 @@
     <row r="274">
       <c r="A274" s="1" t="inlineStr">
         <is>
-          <t>mating projection membrane</t>
+          <t>outer kinetochore</t>
         </is>
       </c>
       <c r="B274" t="n">
@@ -3168,7 +3168,7 @@
     <row r="275">
       <c r="A275" s="1" t="inlineStr">
         <is>
-          <t>nuclear body</t>
+          <t>outer membrane</t>
         </is>
       </c>
       <c r="B275" t="n">
@@ -3178,7 +3178,7 @@
     <row r="276">
       <c r="A276" s="1" t="inlineStr">
         <is>
-          <t>lateral element</t>
+          <t>nuclear pore linkers</t>
         </is>
       </c>
       <c r="B276" t="n">
@@ -3188,7 +3188,7 @@
     <row r="277">
       <c r="A277" s="1" t="inlineStr">
         <is>
-          <t>cortical microtubule plus-end</t>
+          <t>extracellular matrix</t>
         </is>
       </c>
       <c r="B277" t="n">
@@ -3198,7 +3198,7 @@
     <row r="278">
       <c r="A278" s="1" t="inlineStr">
         <is>
-          <t>integral component of organelle membrane</t>
+          <t>nuclear body</t>
         </is>
       </c>
       <c r="B278" t="n">
@@ -3208,7 +3208,7 @@
     <row r="279">
       <c r="A279" s="1" t="inlineStr">
         <is>
-          <t>heterochromatin</t>
+          <t>Golgi cisterna membrane</t>
         </is>
       </c>
       <c r="B279" t="n">
@@ -3218,7 +3218,7 @@
     <row r="280">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>nucleolar preribosome</t>
+          <t>mating projection membrane</t>
         </is>
       </c>
       <c r="B280" t="n">
@@ -3228,7 +3228,7 @@
     <row r="281">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>autophagosome membrane</t>
+          <t>chitosome</t>
         </is>
       </c>
       <c r="B281" t="n">
@@ -3238,7 +3238,7 @@
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>nuclear pore linkers</t>
+          <t>lytic vacuole</t>
         </is>
       </c>
       <c r="B282" t="n">
@@ -3248,7 +3248,7 @@
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>extracellular matrix</t>
+          <t>autophagosome membrane</t>
         </is>
       </c>
       <c r="B283" t="n">
@@ -3258,7 +3258,7 @@
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>secretory vesicle</t>
+          <t>plasma membrane of growing cell tip</t>
         </is>
       </c>
       <c r="B284" t="n">
@@ -3268,7 +3268,7 @@
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>preribosome</t>
+          <t>nuclear inclusion body</t>
         </is>
       </c>
       <c r="B285" t="n">
@@ -3278,7 +3278,7 @@
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>chitosome</t>
+          <t>chromosome, centromeric core domain</t>
         </is>
       </c>
       <c r="B286" t="n">
@@ -3288,7 +3288,7 @@
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>integral component of endosome membrane</t>
+          <t>integral component of lumenal side of endoplasmic reticulum membrane</t>
         </is>
       </c>
       <c r="B287" t="n">
@@ -3298,7 +3298,7 @@
     <row r="288">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>integral component of lumenal side of endoplasmic reticulum membrane</t>
+          <t>nucleolar preribosome</t>
         </is>
       </c>
       <c r="B288" t="n">
@@ -3308,7 +3308,7 @@
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>trans-Golgi network membrane</t>
+          <t>organelle membrane</t>
         </is>
       </c>
       <c r="B289" t="n">
@@ -3318,7 +3318,7 @@
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>host cell viral assembly compartment</t>
+          <t>transverse filament</t>
         </is>
       </c>
       <c r="B290" t="n">
@@ -3328,7 +3328,7 @@
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>prospore septin filament array</t>
+          <t>DNA replication termination region</t>
         </is>
       </c>
       <c r="B291" t="n">
@@ -3338,7 +3338,7 @@
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>extrinsic component of matrix side of mitochondrial inner membrane</t>
+          <t>endoplasmic reticulum-Golgi intermediate compartment membrane</t>
         </is>
       </c>
       <c r="B292" t="n">
@@ -3348,7 +3348,7 @@
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>retrotransposon nucleocapsid</t>
+          <t>intermediate filament</t>
         </is>
       </c>
       <c r="B293" t="n">
@@ -3358,7 +3358,7 @@
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>eisosome membrane domain/MCC</t>
+          <t>host cell viral assembly compartment</t>
         </is>
       </c>
       <c r="B294" t="n">
@@ -3368,7 +3368,7 @@
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>integral component of vacuolar membrane</t>
+          <t>cytoplasmic side of endosome membrane</t>
         </is>
       </c>
       <c r="B295" t="n">
@@ -3378,7 +3378,7 @@
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>trans-Golgi network transport vesicle membrane</t>
+          <t>organelle membrane contact site</t>
         </is>
       </c>
       <c r="B296" t="n">
@@ -3388,7 +3388,7 @@
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>endoplasmic reticulum quality control compartment</t>
+          <t>prespliceosome</t>
         </is>
       </c>
       <c r="B297" t="n">
@@ -3398,7 +3398,7 @@
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>endoplasmic reticulum-Golgi intermediate compartment membrane</t>
+          <t>retrotransposon nucleocapsid</t>
         </is>
       </c>
       <c r="B298" t="n">
@@ -3408,7 +3408,7 @@
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>cytoplasmic side of endosome membrane</t>
+          <t>eisosome membrane domain/MCC</t>
         </is>
       </c>
       <c r="B299" t="n">
@@ -3418,7 +3418,7 @@
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>Cvt vesicle membrane</t>
+          <t>ascus lipid droplet</t>
         </is>
       </c>
       <c r="B300" t="n">
@@ -3428,7 +3428,7 @@
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>ruffle membrane</t>
+          <t>trans-Golgi network membrane</t>
         </is>
       </c>
       <c r="B301" t="n">
@@ -3448,7 +3448,7 @@
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>transverse filament</t>
+          <t>extrinsic component of nuclear outer membrane</t>
         </is>
       </c>
       <c r="B303" t="n">
@@ -3458,7 +3458,7 @@
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>DNA replication termination region</t>
+          <t>extrinsic component of matrix side of mitochondrial inner membrane</t>
         </is>
       </c>
       <c r="B304" t="n">
@@ -3468,7 +3468,7 @@
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>prespliceosome</t>
+          <t>trans-Golgi network transport vesicle membrane</t>
         </is>
       </c>
       <c r="B305" t="n">
@@ -3488,7 +3488,7 @@
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>extrinsic component of nuclear outer membrane</t>
+          <t>perinuclear endoplasmic reticulum membrane</t>
         </is>
       </c>
       <c r="B307" t="n">
@@ -3498,7 +3498,7 @@
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>organelle membrane contact site</t>
+          <t>ruffle membrane</t>
         </is>
       </c>
       <c r="B308" t="n">
@@ -3508,7 +3508,7 @@
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>perinuclear endoplasmic reticulum membrane</t>
+          <t>endoplasmic reticulum quality control compartment</t>
         </is>
       </c>
       <c r="B309" t="n">
@@ -3518,7 +3518,7 @@
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>ascus lipid droplet</t>
+          <t>prospore septin filament array</t>
         </is>
       </c>
       <c r="B310" t="n">
@@ -3528,7 +3528,7 @@
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>nuclear replisome</t>
+          <t>primary cell septum</t>
         </is>
       </c>
       <c r="B311" t="n">
@@ -3538,7 +3538,7 @@
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>intermediate filament</t>
+          <t>nuclear replisome</t>
         </is>
       </c>
       <c r="B312" t="n">
@@ -3548,7 +3548,7 @@
     <row r="313">
       <c r="A313" s="1" t="inlineStr">
         <is>
-          <t>cell wall</t>
+          <t>integral component of vacuolar membrane</t>
         </is>
       </c>
       <c r="B313" t="n">
@@ -3558,7 +3558,7 @@
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>organelle membrane</t>
+          <t>cell wall</t>
         </is>
       </c>
       <c r="B314" t="n">
@@ -3568,7 +3568,7 @@
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>primary cell septum</t>
+          <t>Cvt vesicle membrane</t>
         </is>
       </c>
       <c r="B315" t="n">

</xml_diff>

<commit_message>
feat：add more analysis of membrane
</commit_message>
<xml_diff>
--- a/data/all_component_analysis.xlsx
+++ b/data/all_component_analysis.xlsx
@@ -1408,7 +1408,7 @@
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t>eisosome</t>
+          <t>cortical endoplasmic reticulum</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -1418,7 +1418,7 @@
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t>cortical endoplasmic reticulum</t>
+          <t>nuclear pore outer ring</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -1428,7 +1428,7 @@
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t>nuclear pore outer ring</t>
+          <t>eisosome</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -1438,7 +1438,7 @@
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>integral component of peroxisomal membrane</t>
+          <t>cytoplasmic microtubule</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -1458,7 +1458,7 @@
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t>cytoplasmic microtubule</t>
+          <t>integral component of peroxisomal membrane</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -1548,7 +1548,7 @@
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
         <is>
-          <t>proteasome storage granule</t>
+          <t>endoplasmic reticulum lumen</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -1558,7 +1558,7 @@
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
         <is>
-          <t>site of polarized growth</t>
+          <t>proteasome storage granule</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -1568,7 +1568,7 @@
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
         <is>
-          <t>endoplasmic reticulum lumen</t>
+          <t>site of polarized growth</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -1668,7 +1668,7 @@
     <row r="125">
       <c r="A125" s="1" t="inlineStr">
         <is>
-          <t>cellular bud neck contractile ring</t>
+          <t>COP9 signalosome</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -1678,7 +1678,7 @@
     <row r="126">
       <c r="A126" s="1" t="inlineStr">
         <is>
-          <t>U2-type catalytic step 2 spliceosome</t>
+          <t>cellular bud neck contractile ring</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -1688,7 +1688,7 @@
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
         <is>
-          <t>autophagosome</t>
+          <t>condensed chromosome, centromeric region</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -1698,7 +1698,7 @@
     <row r="128">
       <c r="A128" s="1" t="inlineStr">
         <is>
-          <t>condensed chromosome, centromeric region</t>
+          <t>autophagosome</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -1708,7 +1708,7 @@
     <row r="129">
       <c r="A129" s="1" t="inlineStr">
         <is>
-          <t>COP9 signalosome</t>
+          <t>U2-type catalytic step 2 spliceosome</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -1718,7 +1718,7 @@
     <row r="130">
       <c r="A130" s="1" t="inlineStr">
         <is>
-          <t>fungal-type vacuole lumen</t>
+          <t>late endosome membrane</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -1728,7 +1728,7 @@
     <row r="131">
       <c r="A131" s="1" t="inlineStr">
         <is>
-          <t>multivesicular body</t>
+          <t>cellular bud neck septin ring</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -1738,7 +1738,7 @@
     <row r="132">
       <c r="A132" s="1" t="inlineStr">
         <is>
-          <t>cellular bud neck septin ring</t>
+          <t>multivesicular body</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -1748,7 +1748,7 @@
     <row r="133">
       <c r="A133" s="1" t="inlineStr">
         <is>
-          <t>ascospore wall</t>
+          <t>fungal-type vacuole lumen</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -1758,7 +1758,7 @@
     <row r="134">
       <c r="A134" s="1" t="inlineStr">
         <is>
-          <t>late endosome membrane</t>
+          <t>ascospore wall</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -1768,7 +1768,7 @@
     <row r="135">
       <c r="A135" s="1" t="inlineStr">
         <is>
-          <t>microtubule organizing center</t>
+          <t>intrinsic component of membrane</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -1778,7 +1778,7 @@
     <row r="136">
       <c r="A136" s="1" t="inlineStr">
         <is>
-          <t>perinuclear endoplasmic reticulum</t>
+          <t>microtubule organizing center</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -1788,7 +1788,7 @@
     <row r="137">
       <c r="A137" s="1" t="inlineStr">
         <is>
-          <t>intrinsic component of membrane</t>
+          <t>perinuclear endoplasmic reticulum</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -1798,7 +1798,7 @@
     <row r="138">
       <c r="A138" s="1" t="inlineStr">
         <is>
-          <t>nuclear chromosome</t>
+          <t>recycling endosome</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -1808,7 +1808,7 @@
     <row r="139">
       <c r="A139" s="1" t="inlineStr">
         <is>
-          <t>recycling endosome</t>
+          <t>nuclear chromosome</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -1818,7 +1818,7 @@
     <row r="140">
       <c r="A140" s="1" t="inlineStr">
         <is>
-          <t>cellular bud scar</t>
+          <t>nuclear replication fork</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -1828,7 +1828,7 @@
     <row r="141">
       <c r="A141" s="1" t="inlineStr">
         <is>
-          <t>nuclear replication fork</t>
+          <t>cellular bud scar</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -1848,7 +1848,7 @@
     <row r="143">
       <c r="A143" s="1" t="inlineStr">
         <is>
-          <t>mitochondrial envelope</t>
+          <t>nuclear outer membrane-endoplasmic reticulum membrane network</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -1858,7 +1858,7 @@
     <row r="144">
       <c r="A144" s="1" t="inlineStr">
         <is>
-          <t>nuclear outer membrane-endoplasmic reticulum membrane network</t>
+          <t>mitochondrial envelope</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -1888,7 +1888,7 @@
     <row r="147">
       <c r="A147" s="1" t="inlineStr">
         <is>
-          <t>integral component of mitochondrial membrane</t>
+          <t>vacuolar proton-transporting V-type ATPase, V1 domain</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -1898,7 +1898,7 @@
     <row r="148">
       <c r="A148" s="1" t="inlineStr">
         <is>
-          <t>endocytic vesicle</t>
+          <t>integral component of mitochondrial membrane</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -1908,7 +1908,7 @@
     <row r="149">
       <c r="A149" s="1" t="inlineStr">
         <is>
-          <t>cell cortex of cell tip</t>
+          <t>nuclear pore cytoplasmic filaments</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -1918,7 +1918,7 @@
     <row r="150">
       <c r="A150" s="1" t="inlineStr">
         <is>
-          <t>nuclear pore cytoplasmic filaments</t>
+          <t>endocytic vesicle</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -1938,7 +1938,7 @@
     <row r="152">
       <c r="A152" s="1" t="inlineStr">
         <is>
-          <t>vacuolar proton-transporting V-type ATPase, V1 domain</t>
+          <t>cell cortex of cell tip</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -1948,7 +1948,7 @@
     <row r="153">
       <c r="A153" s="1" t="inlineStr">
         <is>
-          <t>respirasome</t>
+          <t>transcriptionally active chromatin</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -1958,7 +1958,7 @@
     <row r="154">
       <c r="A154" s="1" t="inlineStr">
         <is>
-          <t>cytoplasmic vesicle membrane</t>
+          <t>respirasome</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -1968,7 +1968,7 @@
     <row r="155">
       <c r="A155" s="1" t="inlineStr">
         <is>
-          <t>transcriptionally active chromatin</t>
+          <t>cytoplasmic vesicle membrane</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -1988,7 +1988,7 @@
     <row r="157">
       <c r="A157" s="1" t="inlineStr">
         <is>
-          <t>vacuolar proton-transporting V-type ATPase, V0 domain</t>
+          <t>CHRAC</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -1998,7 +1998,7 @@
     <row r="158">
       <c r="A158" s="1" t="inlineStr">
         <is>
-          <t>CHRAC</t>
+          <t>vacuolar proton-transporting V-type ATPase, V0 domain</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -2008,7 +2008,7 @@
     <row r="159">
       <c r="A159" s="1" t="inlineStr">
         <is>
-          <t>nuclear pore nuclear basket</t>
+          <t>vacuole-mitochondrion membrane contact site</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -2028,7 +2028,7 @@
     <row r="161">
       <c r="A161" s="1" t="inlineStr">
         <is>
-          <t>nuclear pore inner ring</t>
+          <t>COPI-coated vesicle</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -2038,7 +2038,7 @@
     <row r="162">
       <c r="A162" s="1" t="inlineStr">
         <is>
-          <t>COPI-coated vesicle</t>
+          <t>nuclear pore inner ring</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -2048,7 +2048,7 @@
     <row r="163">
       <c r="A163" s="1" t="inlineStr">
         <is>
-          <t>vacuole-mitochondrion membrane contact site</t>
+          <t>nuclear pore nuclear basket</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -2058,7 +2058,7 @@
     <row r="164">
       <c r="A164" s="1" t="inlineStr">
         <is>
-          <t>Golgi stack</t>
+          <t>extrinsic component of fungal-type vacuolar membrane</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -2068,7 +2068,7 @@
     <row r="165">
       <c r="A165" s="1" t="inlineStr">
         <is>
-          <t>extrinsic component of fungal-type vacuolar membrane</t>
+          <t>Golgi stack</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -2088,7 +2088,7 @@
     <row r="167">
       <c r="A167" s="1" t="inlineStr">
         <is>
-          <t>actomyosin contractile ring</t>
+          <t>COPI-coated vesicle membrane</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -2098,7 +2098,7 @@
     <row r="168">
       <c r="A168" s="1" t="inlineStr">
         <is>
-          <t>extrinsic component of endoplasmic reticulum membrane</t>
+          <t>transport vesicle</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -2108,7 +2108,7 @@
     <row r="169">
       <c r="A169" s="1" t="inlineStr">
         <is>
-          <t>transport vesicle</t>
+          <t>actomyosin contractile ring</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -2118,7 +2118,7 @@
     <row r="170">
       <c r="A170" s="1" t="inlineStr">
         <is>
-          <t>COPI-coated vesicle membrane</t>
+          <t>extrinsic component of endoplasmic reticulum membrane</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -2128,7 +2128,7 @@
     <row r="171">
       <c r="A171" s="1" t="inlineStr">
         <is>
-          <t>Golgi medial cisterna</t>
+          <t>rDNA heterochromatin</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -2138,7 +2138,7 @@
     <row r="172">
       <c r="A172" s="1" t="inlineStr">
         <is>
-          <t>rDNA heterochromatin</t>
+          <t>Golgi medial cisterna</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -2178,7 +2178,7 @@
     <row r="176">
       <c r="A176" s="1" t="inlineStr">
         <is>
-          <t>endoplasmic reticulum tubular network</t>
+          <t>mating projection</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -2188,7 +2188,7 @@
     <row r="177">
       <c r="A177" s="1" t="inlineStr">
         <is>
-          <t>mating projection</t>
+          <t>endoplasmic reticulum tubular network</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -2198,7 +2198,7 @@
     <row r="178">
       <c r="A178" s="1" t="inlineStr">
         <is>
-          <t>early endosome membrane</t>
+          <t>mitochondrial crista junction</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -2208,7 +2208,7 @@
     <row r="179">
       <c r="A179" s="1" t="inlineStr">
         <is>
-          <t>growing cell tip</t>
+          <t>Golgi cis cisterna</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -2218,7 +2218,7 @@
     <row r="180">
       <c r="A180" s="1" t="inlineStr">
         <is>
-          <t>mitochondrial crista junction</t>
+          <t>early endosome membrane</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -2228,7 +2228,7 @@
     <row r="181">
       <c r="A181" s="1" t="inlineStr">
         <is>
-          <t>Golgi cis cisterna</t>
+          <t>proton-transporting V-type ATPase, V0 domain</t>
         </is>
       </c>
       <c r="B181" t="n">
@@ -2238,7 +2238,7 @@
     <row r="182">
       <c r="A182" s="1" t="inlineStr">
         <is>
-          <t>Golgi trans cisterna</t>
+          <t>intrinsic component of mitochondrial inner membrane</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -2248,7 +2248,7 @@
     <row r="183">
       <c r="A183" s="1" t="inlineStr">
         <is>
-          <t>mitochondrial proton-transporting ATP synthase, stator stalk</t>
+          <t>growing cell tip</t>
         </is>
       </c>
       <c r="B183" t="n">
@@ -2258,7 +2258,7 @@
     <row r="184">
       <c r="A184" s="1" t="inlineStr">
         <is>
-          <t>clathrin-coated vesicle membrane</t>
+          <t>mitochondrial proton-transporting ATP synthase, stator stalk</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -2268,7 +2268,7 @@
     <row r="185">
       <c r="A185" s="1" t="inlineStr">
         <is>
-          <t>phagophore</t>
+          <t>clathrin-coated vesicle membrane</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -2278,7 +2278,7 @@
     <row r="186">
       <c r="A186" s="1" t="inlineStr">
         <is>
-          <t>vacuole-isolation membrane contact site</t>
+          <t>phagophore</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -2288,7 +2288,7 @@
     <row r="187">
       <c r="A187" s="1" t="inlineStr">
         <is>
-          <t>intrinsic component of mitochondrial inner membrane</t>
+          <t>Golgi trans cisterna</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -2298,7 +2298,7 @@
     <row r="188">
       <c r="A188" s="1" t="inlineStr">
         <is>
-          <t>proton-transporting V-type ATPase, V0 domain</t>
+          <t>vacuole-isolation membrane contact site</t>
         </is>
       </c>
       <c r="B188" t="n">
@@ -2308,7 +2308,7 @@
     <row r="189">
       <c r="A189" s="1" t="inlineStr">
         <is>
-          <t>cytosolic ribosome</t>
+          <t>prospore membrane leading edge</t>
         </is>
       </c>
       <c r="B189" t="n">
@@ -2318,7 +2318,7 @@
     <row r="190">
       <c r="A190" s="1" t="inlineStr">
         <is>
-          <t>phagocytic vesicle</t>
+          <t>signal recognition particle</t>
         </is>
       </c>
       <c r="B190" t="n">
@@ -2328,7 +2328,7 @@
     <row r="191">
       <c r="A191" s="1" t="inlineStr">
         <is>
-          <t>nuclear microtubule</t>
+          <t>phagocytic vesicle</t>
         </is>
       </c>
       <c r="B191" t="n">
@@ -2348,7 +2348,7 @@
     <row r="193">
       <c r="A193" s="1" t="inlineStr">
         <is>
-          <t>mitochondrial proton-transporting ATP synthase, catalytic core</t>
+          <t>nuclear microtubule</t>
         </is>
       </c>
       <c r="B193" t="n">
@@ -2358,7 +2358,7 @@
     <row r="194">
       <c r="A194" s="1" t="inlineStr">
         <is>
-          <t>prospore membrane leading edge</t>
+          <t>condensed chromosome</t>
         </is>
       </c>
       <c r="B194" t="n">
@@ -2368,7 +2368,7 @@
     <row r="195">
       <c r="A195" s="1" t="inlineStr">
         <is>
-          <t>mitochondrial respirasome</t>
+          <t>mitochondrial proton-transporting ATP synthase, catalytic core</t>
         </is>
       </c>
       <c r="B195" t="n">
@@ -2378,7 +2378,7 @@
     <row r="196">
       <c r="A196" s="1" t="inlineStr">
         <is>
-          <t>condensed chromosome</t>
+          <t>cytosolic ribosome</t>
         </is>
       </c>
       <c r="B196" t="n">
@@ -2388,7 +2388,7 @@
     <row r="197">
       <c r="A197" s="1" t="inlineStr">
         <is>
-          <t>signal recognition particle</t>
+          <t>mitochondrial respirasome</t>
         </is>
       </c>
       <c r="B197" t="n">
@@ -2398,7 +2398,7 @@
     <row r="198">
       <c r="A198" s="1" t="inlineStr">
         <is>
-          <t>cell wall-bounded periplasmic space</t>
+          <t>extrinsic component of vacuolar membrane</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -2408,7 +2408,7 @@
     <row r="199">
       <c r="A199" s="1" t="inlineStr">
         <is>
-          <t>extrinsic component of vacuolar membrane</t>
+          <t>cell wall-bounded periplasmic space</t>
         </is>
       </c>
       <c r="B199" t="n">
@@ -2418,7 +2418,7 @@
     <row r="200">
       <c r="A200" s="1" t="inlineStr">
         <is>
-          <t>cellular bud neck septin collar</t>
+          <t>vacuolar lumen</t>
         </is>
       </c>
       <c r="B200" t="n">
@@ -2428,7 +2428,7 @@
     <row r="201">
       <c r="A201" s="1" t="inlineStr">
         <is>
-          <t>vacuolar lumen</t>
+          <t>cytoplasmic side of plasma membrane</t>
         </is>
       </c>
       <c r="B201" t="n">
@@ -2438,7 +2438,7 @@
     <row r="202">
       <c r="A202" s="1" t="inlineStr">
         <is>
-          <t>proteasome regulatory particle</t>
+          <t>spore wall</t>
         </is>
       </c>
       <c r="B202" t="n">
@@ -2448,7 +2448,7 @@
     <row r="203">
       <c r="A203" s="1" t="inlineStr">
         <is>
-          <t>spore wall</t>
+          <t>extrinsic component of plasma membrane</t>
         </is>
       </c>
       <c r="B203" t="n">
@@ -2458,7 +2458,7 @@
     <row r="204">
       <c r="A204" s="1" t="inlineStr">
         <is>
-          <t>cytoplasmic side of plasma membrane</t>
+          <t>proteasome regulatory particle</t>
         </is>
       </c>
       <c r="B204" t="n">
@@ -2468,7 +2468,7 @@
     <row r="205">
       <c r="A205" s="1" t="inlineStr">
         <is>
-          <t>extrinsic component of plasma membrane</t>
+          <t>cellular bud neck septin collar</t>
         </is>
       </c>
       <c r="B205" t="n">
@@ -2478,7 +2478,7 @@
     <row r="206">
       <c r="A206" s="1" t="inlineStr">
         <is>
-          <t>nuclear outer membrane</t>
+          <t>mating projection base</t>
         </is>
       </c>
       <c r="B206" t="n">
@@ -2488,7 +2488,7 @@
     <row r="207">
       <c r="A207" s="1" t="inlineStr">
         <is>
-          <t>mitochondrial chromosome</t>
+          <t>mitochondrial inner boundary membrane</t>
         </is>
       </c>
       <c r="B207" t="n">
@@ -2498,7 +2498,7 @@
     <row r="208">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>mitochondrial inner boundary membrane</t>
+          <t>kinetochore microtubule</t>
         </is>
       </c>
       <c r="B208" t="n">
@@ -2508,7 +2508,7 @@
     <row r="209">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>mating projection base</t>
+          <t>mitochondrial proton-transporting ATP synthase, central stalk</t>
         </is>
       </c>
       <c r="B209" t="n">
@@ -2518,7 +2518,7 @@
     <row r="210">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>extrinsic component of cytoplasmic side of plasma membrane</t>
+          <t>mitochondrial chromosome</t>
         </is>
       </c>
       <c r="B210" t="n">
@@ -2528,7 +2528,7 @@
     <row r="211">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>division septum</t>
+          <t>nuclear outer membrane</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -2538,7 +2538,7 @@
     <row r="212">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>nucleolar chromatin</t>
+          <t>extrinsic component of cytoplasmic side of plasma membrane</t>
         </is>
       </c>
       <c r="B212" t="n">
@@ -2548,7 +2548,7 @@
     <row r="213">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>medial cortex</t>
+          <t>nucleolar chromatin</t>
         </is>
       </c>
       <c r="B213" t="n">
@@ -2558,7 +2558,7 @@
     <row r="214">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>kinetochore microtubule</t>
+          <t>division septum</t>
         </is>
       </c>
       <c r="B214" t="n">
@@ -2578,7 +2578,7 @@
     <row r="216">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>mitochondrial proton-transporting ATP synthase, central stalk</t>
+          <t>medial cortex</t>
         </is>
       </c>
       <c r="B216" t="n">
@@ -2588,7 +2588,7 @@
     <row r="217">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>nuclear matrix</t>
+          <t>nuclear envelope lumen</t>
         </is>
       </c>
       <c r="B217" t="n">
@@ -2598,7 +2598,7 @@
     <row r="218">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>anchored component of plasma membrane</t>
+          <t>mitochondrial degradosome</t>
         </is>
       </c>
       <c r="B218" t="n">
@@ -2608,7 +2608,7 @@
     <row r="219">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>mitochondria-associated endoplasmic reticulum membrane</t>
+          <t>nuclear matrix</t>
         </is>
       </c>
       <c r="B219" t="n">
@@ -2618,7 +2618,7 @@
     <row r="220">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>mitochondrial degradosome</t>
+          <t>polysomal ribosome</t>
         </is>
       </c>
       <c r="B220" t="n">
@@ -2628,7 +2628,7 @@
     <row r="221">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>nuclear envelope lumen</t>
+          <t>mitochondria-associated endoplasmic reticulum membrane</t>
         </is>
       </c>
       <c r="B221" t="n">
@@ -2638,7 +2638,7 @@
     <row r="222">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>membrane-bounded organelle</t>
+          <t>anchored component of plasma membrane</t>
         </is>
       </c>
       <c r="B222" t="n">
@@ -2648,7 +2648,7 @@
     <row r="223">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>polysomal ribosome</t>
+          <t>membrane-bounded organelle</t>
         </is>
       </c>
       <c r="B223" t="n">
@@ -2658,7 +2658,7 @@
     <row r="224">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>RNA polymerase II, holoenzyme</t>
+          <t>nucleoid</t>
         </is>
       </c>
       <c r="B224" t="n">
@@ -2668,7 +2668,7 @@
     <row r="225">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>mitotic actomyosin contractile ring</t>
+          <t>integral component of nuclear inner membrane</t>
         </is>
       </c>
       <c r="B225" t="n">
@@ -2678,7 +2678,7 @@
     <row r="226">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>eisosome filament</t>
+          <t>septin filament array</t>
         </is>
       </c>
       <c r="B226" t="n">
@@ -2688,7 +2688,7 @@
     <row r="227">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>trans-Golgi network transport vesicle</t>
+          <t>matrix side of mitochondrial inner membrane</t>
         </is>
       </c>
       <c r="B227" t="n">
@@ -2698,7 +2698,7 @@
     <row r="228">
       <c r="A228" s="1" t="inlineStr">
         <is>
-          <t>mitochondrial crista</t>
+          <t>CENP-A containing nucleosome</t>
         </is>
       </c>
       <c r="B228" t="n">
@@ -2708,7 +2708,7 @@
     <row r="229">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>matrix side of mitochondrial inner membrane</t>
+          <t>extrinsic component of mitochondrial outer membrane</t>
         </is>
       </c>
       <c r="B229" t="n">
@@ -2718,7 +2718,7 @@
     <row r="230">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>integral component of nuclear inner membrane</t>
+          <t>tubular endosome</t>
         </is>
       </c>
       <c r="B230" t="n">
@@ -2728,7 +2728,7 @@
     <row r="231">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>integral component of nuclear outer membrane</t>
+          <t>mitochondrial crista</t>
         </is>
       </c>
       <c r="B231" t="n">
@@ -2738,7 +2738,7 @@
     <row r="232">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>extrinsic component of mitochondrial outer membrane</t>
+          <t>trans-Golgi network transport vesicle</t>
         </is>
       </c>
       <c r="B232" t="n">
@@ -2748,7 +2748,7 @@
     <row r="233">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>septin filament array</t>
+          <t>eisosome filament</t>
         </is>
       </c>
       <c r="B233" t="n">
@@ -2758,7 +2758,7 @@
     <row r="234">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>proton-transporting V-type ATPase, V1 domain</t>
+          <t>cell cortex of growing cell tip</t>
         </is>
       </c>
       <c r="B234" t="n">
@@ -2768,7 +2768,7 @@
     <row r="235">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>tubular endosome</t>
+          <t>mating projection tip membrane</t>
         </is>
       </c>
       <c r="B235" t="n">
@@ -2778,7 +2778,7 @@
     <row r="236">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>mating-type region heterochromatin</t>
+          <t>mitotic actomyosin contractile ring</t>
         </is>
       </c>
       <c r="B236" t="n">
@@ -2788,7 +2788,7 @@
     <row r="237">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>cell cortex of growing cell tip</t>
+          <t>proton-transporting V-type ATPase, V1 domain</t>
         </is>
       </c>
       <c r="B237" t="n">
@@ -2798,7 +2798,7 @@
     <row r="238">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>CENP-A containing nucleosome</t>
+          <t>integral component of nuclear outer membrane</t>
         </is>
       </c>
       <c r="B238" t="n">
@@ -2808,7 +2808,7 @@
     <row r="239">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>extrinsic component of intraperoxisomal membrane</t>
+          <t>RNA polymerase II, holoenzyme</t>
         </is>
       </c>
       <c r="B239" t="n">
@@ -2818,7 +2818,7 @@
     <row r="240">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>mating projection tip membrane</t>
+          <t>extrinsic component of intraperoxisomal membrane</t>
         </is>
       </c>
       <c r="B240" t="n">
@@ -2828,7 +2828,7 @@
     <row r="241">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>nucleoid</t>
+          <t>mating-type region heterochromatin</t>
         </is>
       </c>
       <c r="B241" t="n">
@@ -2838,7 +2838,7 @@
     <row r="242">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>astral microtubule</t>
+          <t>integral component of cytoplasmic side of endoplasmic reticulum membrane</t>
         </is>
       </c>
       <c r="B242" t="n">
@@ -2848,7 +2848,7 @@
     <row r="243">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>replisome</t>
+          <t>multivesicular body membrane</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -2858,7 +2858,7 @@
     <row r="244">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>multivesicular body membrane</t>
+          <t>cytoplasmic side of membrane</t>
         </is>
       </c>
       <c r="B244" t="n">
@@ -2868,7 +2868,7 @@
     <row r="245">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>cis-Golgi network membrane</t>
+          <t>clathrin coat of coated pit</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -2878,7 +2878,7 @@
     <row r="246">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>Golgi cisterna</t>
+          <t>mitotic actomyosin contractile ring, proximal layer</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -2888,7 +2888,7 @@
     <row r="247">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>transport vesicle membrane</t>
+          <t>Golgi-associated vesicle</t>
         </is>
       </c>
       <c r="B247" t="n">
@@ -2898,7 +2898,7 @@
     <row r="248">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>intrinsic component of endoplasmic reticulum membrane</t>
+          <t>cis-Golgi network membrane</t>
         </is>
       </c>
       <c r="B248" t="n">
@@ -2918,7 +2918,7 @@
     <row r="250">
       <c r="A250" s="1" t="inlineStr">
         <is>
-          <t>nuclear speck</t>
+          <t>intrinsic component of the cytoplasmic side of the plasma membrane</t>
         </is>
       </c>
       <c r="B250" t="n">
@@ -2928,7 +2928,7 @@
     <row r="251">
       <c r="A251" s="1" t="inlineStr">
         <is>
-          <t>Golgi-associated vesicle</t>
+          <t>clathrin coat of trans-Golgi network vesicle</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -2938,7 +2938,7 @@
     <row r="252">
       <c r="A252" s="1" t="inlineStr">
         <is>
-          <t>mitotic actomyosin contractile ring, proximal layer</t>
+          <t>nuclear speck</t>
         </is>
       </c>
       <c r="B252" t="n">
@@ -2948,7 +2948,7 @@
     <row r="253">
       <c r="A253" s="1" t="inlineStr">
         <is>
-          <t>anchored component of the cytoplasmic side of the plasma membrane</t>
+          <t>ascospore-type prospore</t>
         </is>
       </c>
       <c r="B253" t="n">
@@ -2958,7 +2958,7 @@
     <row r="254">
       <c r="A254" s="1" t="inlineStr">
         <is>
-          <t>clathrin coat of coated pit</t>
+          <t>astral microtubule</t>
         </is>
       </c>
       <c r="B254" t="n">
@@ -2968,7 +2968,7 @@
     <row r="255">
       <c r="A255" s="1" t="inlineStr">
         <is>
-          <t>intrinsic component of the cytoplasmic side of the plasma membrane</t>
+          <t>replisome</t>
         </is>
       </c>
       <c r="B255" t="n">
@@ -2978,7 +2978,7 @@
     <row r="256">
       <c r="A256" s="1" t="inlineStr">
         <is>
-          <t>integral component of cytoplasmic side of endoplasmic reticulum membrane</t>
+          <t>anchored component of the cytoplasmic side of the plasma membrane</t>
         </is>
       </c>
       <c r="B256" t="n">
@@ -2988,7 +2988,7 @@
     <row r="257">
       <c r="A257" s="1" t="inlineStr">
         <is>
-          <t>ascospore-type prospore</t>
+          <t>Golgi cisterna</t>
         </is>
       </c>
       <c r="B257" t="n">
@@ -2998,7 +2998,7 @@
     <row r="258">
       <c r="A258" s="1" t="inlineStr">
         <is>
-          <t>cytoplasmic side of membrane</t>
+          <t>transport vesicle membrane</t>
         </is>
       </c>
       <c r="B258" t="n">
@@ -3008,7 +3008,7 @@
     <row r="259">
       <c r="A259" s="1" t="inlineStr">
         <is>
-          <t>clathrin coat of trans-Golgi network vesicle</t>
+          <t>intrinsic component of endoplasmic reticulum membrane</t>
         </is>
       </c>
       <c r="B259" t="n">
@@ -3018,7 +3018,7 @@
     <row r="260">
       <c r="A260" s="1" t="inlineStr">
         <is>
-          <t>P granule</t>
+          <t>polar microtubule</t>
         </is>
       </c>
       <c r="B260" t="n">
@@ -3028,7 +3028,7 @@
     <row r="261">
       <c r="A261" s="1" t="inlineStr">
         <is>
-          <t>integral component of organelle membrane</t>
+          <t>autophagosome membrane</t>
         </is>
       </c>
       <c r="B261" t="n">
@@ -3048,7 +3048,7 @@
     <row r="263">
       <c r="A263" s="1" t="inlineStr">
         <is>
-          <t>intrinsic component of vacuolar membrane</t>
+          <t>replication compartment</t>
         </is>
       </c>
       <c r="B263" t="n">
@@ -3058,7 +3058,7 @@
     <row r="264">
       <c r="A264" s="1" t="inlineStr">
         <is>
-          <t>cellular birth scar</t>
+          <t>nuclear pore linkers</t>
         </is>
       </c>
       <c r="B264" t="n">
@@ -3068,7 +3068,7 @@
     <row r="265">
       <c r="A265" s="1" t="inlineStr">
         <is>
-          <t>integral component of endosome membrane</t>
+          <t>chromosome, centromeric core domain</t>
         </is>
       </c>
       <c r="B265" t="n">
@@ -3078,7 +3078,7 @@
     <row r="266">
       <c r="A266" s="1" t="inlineStr">
         <is>
-          <t>replication compartment</t>
+          <t>lateral element</t>
         </is>
       </c>
       <c r="B266" t="n">
@@ -3088,7 +3088,7 @@
     <row r="267">
       <c r="A267" s="1" t="inlineStr">
         <is>
-          <t>preribosome</t>
+          <t>lytic vacuole</t>
         </is>
       </c>
       <c r="B267" t="n">
@@ -3098,7 +3098,7 @@
     <row r="268">
       <c r="A268" s="1" t="inlineStr">
         <is>
-          <t>secretory vesicle</t>
+          <t>integral component of lumenal side of endoplasmic reticulum membrane</t>
         </is>
       </c>
       <c r="B268" t="n">
@@ -3118,7 +3118,7 @@
     <row r="270">
       <c r="A270" s="1" t="inlineStr">
         <is>
-          <t>lateral element</t>
+          <t>chitosome</t>
         </is>
       </c>
       <c r="B270" t="n">
@@ -3128,7 +3128,7 @@
     <row r="271">
       <c r="A271" s="1" t="inlineStr">
         <is>
-          <t>polar microtubule</t>
+          <t>preribosome</t>
         </is>
       </c>
       <c r="B271" t="n">
@@ -3138,7 +3138,7 @@
     <row r="272">
       <c r="A272" s="1" t="inlineStr">
         <is>
-          <t>heterochromatin</t>
+          <t>outer membrane</t>
         </is>
       </c>
       <c r="B272" t="n">
@@ -3148,7 +3148,7 @@
     <row r="273">
       <c r="A273" s="1" t="inlineStr">
         <is>
-          <t>2-micrometer circle DNA</t>
+          <t>plasma membrane of growing cell tip</t>
         </is>
       </c>
       <c r="B273" t="n">
@@ -3168,7 +3168,7 @@
     <row r="275">
       <c r="A275" s="1" t="inlineStr">
         <is>
-          <t>outer membrane</t>
+          <t>2-micrometer circle DNA</t>
         </is>
       </c>
       <c r="B275" t="n">
@@ -3178,7 +3178,7 @@
     <row r="276">
       <c r="A276" s="1" t="inlineStr">
         <is>
-          <t>nuclear pore linkers</t>
+          <t>mating projection membrane</t>
         </is>
       </c>
       <c r="B276" t="n">
@@ -3188,7 +3188,7 @@
     <row r="277">
       <c r="A277" s="1" t="inlineStr">
         <is>
-          <t>extracellular matrix</t>
+          <t>integral component of organelle membrane</t>
         </is>
       </c>
       <c r="B277" t="n">
@@ -3198,7 +3198,7 @@
     <row r="278">
       <c r="A278" s="1" t="inlineStr">
         <is>
-          <t>nuclear body</t>
+          <t>cellular birth scar</t>
         </is>
       </c>
       <c r="B278" t="n">
@@ -3208,7 +3208,7 @@
     <row r="279">
       <c r="A279" s="1" t="inlineStr">
         <is>
-          <t>Golgi cisterna membrane</t>
+          <t>heterochromatin</t>
         </is>
       </c>
       <c r="B279" t="n">
@@ -3218,7 +3218,7 @@
     <row r="280">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>mating projection membrane</t>
+          <t>extracellular matrix</t>
         </is>
       </c>
       <c r="B280" t="n">
@@ -3228,7 +3228,7 @@
     <row r="281">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>chitosome</t>
+          <t>intrinsic component of vacuolar membrane</t>
         </is>
       </c>
       <c r="B281" t="n">
@@ -3238,7 +3238,7 @@
     <row r="282">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>lytic vacuole</t>
+          <t>P granule</t>
         </is>
       </c>
       <c r="B282" t="n">
@@ -3248,7 +3248,7 @@
     <row r="283">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>autophagosome membrane</t>
+          <t>secretory vesicle</t>
         </is>
       </c>
       <c r="B283" t="n">
@@ -3258,7 +3258,7 @@
     <row r="284">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>plasma membrane of growing cell tip</t>
+          <t>integral component of endosome membrane</t>
         </is>
       </c>
       <c r="B284" t="n">
@@ -3268,7 +3268,7 @@
     <row r="285">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>nuclear inclusion body</t>
+          <t>nuclear body</t>
         </is>
       </c>
       <c r="B285" t="n">
@@ -3278,7 +3278,7 @@
     <row r="286">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>chromosome, centromeric core domain</t>
+          <t>nuclear inclusion body</t>
         </is>
       </c>
       <c r="B286" t="n">
@@ -3288,7 +3288,7 @@
     <row r="287">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>integral component of lumenal side of endoplasmic reticulum membrane</t>
+          <t>Golgi cisterna membrane</t>
         </is>
       </c>
       <c r="B287" t="n">
@@ -3308,7 +3308,7 @@
     <row r="289">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>organelle membrane</t>
+          <t>Cvt vesicle membrane</t>
         </is>
       </c>
       <c r="B289" t="n">
@@ -3318,7 +3318,7 @@
     <row r="290">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>transverse filament</t>
+          <t>nuclear replisome</t>
         </is>
       </c>
       <c r="B290" t="n">
@@ -3328,7 +3328,7 @@
     <row r="291">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>DNA replication termination region</t>
+          <t>transverse filament</t>
         </is>
       </c>
       <c r="B291" t="n">
@@ -3338,7 +3338,7 @@
     <row r="292">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>endoplasmic reticulum-Golgi intermediate compartment membrane</t>
+          <t>primary cell septum</t>
         </is>
       </c>
       <c r="B292" t="n">
@@ -3348,7 +3348,7 @@
     <row r="293">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>intermediate filament</t>
+          <t>DNA replication termination region</t>
         </is>
       </c>
       <c r="B293" t="n">
@@ -3358,7 +3358,7 @@
     <row r="294">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>host cell viral assembly compartment</t>
+          <t>endocytic patch</t>
         </is>
       </c>
       <c r="B294" t="n">
@@ -3368,7 +3368,7 @@
     <row r="295">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>cytoplasmic side of endosome membrane</t>
+          <t>retrotransposon nucleocapsid</t>
         </is>
       </c>
       <c r="B295" t="n">
@@ -3378,7 +3378,7 @@
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>organelle membrane contact site</t>
+          <t>intermediate filament</t>
         </is>
       </c>
       <c r="B296" t="n">
@@ -3388,7 +3388,7 @@
     <row r="297">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>prespliceosome</t>
+          <t>ascus lipid droplet</t>
         </is>
       </c>
       <c r="B297" t="n">
@@ -3398,7 +3398,7 @@
     <row r="298">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>retrotransposon nucleocapsid</t>
+          <t>trans-Golgi network transport vesicle membrane</t>
         </is>
       </c>
       <c r="B298" t="n">
@@ -3408,7 +3408,7 @@
     <row r="299">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>eisosome membrane domain/MCC</t>
+          <t>host cell viral assembly compartment</t>
         </is>
       </c>
       <c r="B299" t="n">
@@ -3418,7 +3418,7 @@
     <row r="300">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>ascus lipid droplet</t>
+          <t>organelle membrane contact site</t>
         </is>
       </c>
       <c r="B300" t="n">
@@ -3428,7 +3428,7 @@
     <row r="301">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>trans-Golgi network membrane</t>
+          <t>organelle membrane</t>
         </is>
       </c>
       <c r="B301" t="n">
@@ -3438,7 +3438,7 @@
     <row r="302">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>endocytic patch</t>
+          <t>ruffle membrane</t>
         </is>
       </c>
       <c r="B302" t="n">
@@ -3448,7 +3448,7 @@
     <row r="303">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>extrinsic component of nuclear outer membrane</t>
+          <t>endoplasmic reticulum-Golgi intermediate compartment membrane</t>
         </is>
       </c>
       <c r="B303" t="n">
@@ -3458,7 +3458,7 @@
     <row r="304">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>extrinsic component of matrix side of mitochondrial inner membrane</t>
+          <t>cell wall</t>
         </is>
       </c>
       <c r="B304" t="n">
@@ -3468,7 +3468,7 @@
     <row r="305">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>trans-Golgi network transport vesicle membrane</t>
+          <t>endoplasmic reticulum quality control compartment</t>
         </is>
       </c>
       <c r="B305" t="n">
@@ -3488,7 +3488,7 @@
     <row r="307">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>perinuclear endoplasmic reticulum membrane</t>
+          <t>extrinsic component of nuclear outer membrane</t>
         </is>
       </c>
       <c r="B307" t="n">
@@ -3498,7 +3498,7 @@
     <row r="308">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>ruffle membrane</t>
+          <t>eisosome membrane domain/MCC</t>
         </is>
       </c>
       <c r="B308" t="n">
@@ -3508,7 +3508,7 @@
     <row r="309">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>endoplasmic reticulum quality control compartment</t>
+          <t>cytoplasmic side of endosome membrane</t>
         </is>
       </c>
       <c r="B309" t="n">
@@ -3518,7 +3518,7 @@
     <row r="310">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>prospore septin filament array</t>
+          <t>extrinsic component of matrix side of mitochondrial inner membrane</t>
         </is>
       </c>
       <c r="B310" t="n">
@@ -3528,7 +3528,7 @@
     <row r="311">
       <c r="A311" s="1" t="inlineStr">
         <is>
-          <t>primary cell septum</t>
+          <t>prespliceosome</t>
         </is>
       </c>
       <c r="B311" t="n">
@@ -3538,7 +3538,7 @@
     <row r="312">
       <c r="A312" s="1" t="inlineStr">
         <is>
-          <t>nuclear replisome</t>
+          <t>trans-Golgi network membrane</t>
         </is>
       </c>
       <c r="B312" t="n">
@@ -3558,7 +3558,7 @@
     <row r="314">
       <c r="A314" s="1" t="inlineStr">
         <is>
-          <t>cell wall</t>
+          <t>perinuclear endoplasmic reticulum membrane</t>
         </is>
       </c>
       <c r="B314" t="n">
@@ -3568,7 +3568,7 @@
     <row r="315">
       <c r="A315" s="1" t="inlineStr">
         <is>
-          <t>Cvt vesicle membrane</t>
+          <t>prospore septin filament array</t>
         </is>
       </c>
       <c r="B315" t="n">

</xml_diff>